<commit_message>
quick change month by month
</commit_message>
<xml_diff>
--- a/Month_by_Month.xlsx
+++ b/Month_by_Month.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leech\Documents\DATA_Labs\Capstone_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04DAFBAE-31B1-481B-980D-7B73C134C9F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C4203FD-78A7-4464-A751-11866E2E2457}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="4" xr2:uid="{5487F7B6-664A-4C52-988B-A77C01D68399}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="25820" windowHeight="15500" activeTab="4" xr2:uid="{5487F7B6-664A-4C52-988B-A77C01D68399}"/>
   </bookViews>
   <sheets>
     <sheet name="Connecticut" sheetId="3" r:id="rId1"/>
@@ -41,11 +41,11 @@
   </definedNames>
   <calcPr calcId="0"/>
   <pivotCaches>
-    <pivotCache cacheId="305" r:id="rId6"/>
-    <pivotCache cacheId="395" r:id="rId7"/>
-    <pivotCache cacheId="407" r:id="rId8"/>
-    <pivotCache cacheId="419" r:id="rId9"/>
-    <pivotCache cacheId="518" r:id="rId10"/>
+    <pivotCache cacheId="809" r:id="rId6"/>
+    <pivotCache cacheId="845" r:id="rId7"/>
+    <pivotCache cacheId="848" r:id="rId8"/>
+    <pivotCache cacheId="851" r:id="rId9"/>
+    <pivotCache cacheId="854" r:id="rId10"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{876F7934-8845-4945-9796-88D515C7AA90}">
@@ -819,7 +819,1351 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="511">
+  <dxfs count="735">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -4094,16 +5438,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>32008.85</c:v>
+                  <c:v>30369.64</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>39754.07</c:v>
+                  <c:v>49175.79</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>48142.95</c:v>
+                  <c:v>44890.28</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>60671.67</c:v>
+                  <c:v>71032.14</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4843,16 +6187,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>32008.85</c:v>
+                  <c:v>30369.64</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>39754.07</c:v>
+                  <c:v>49175.79</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>48142.95</c:v>
+                  <c:v>44890.28</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>60671.67</c:v>
+                  <c:v>71032.14</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5270,16 +6614,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>687382.03</c:v>
+                  <c:v>56250.74</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1044157.05</c:v>
+                  <c:v>90818.8</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1046676.37</c:v>
+                  <c:v>89422.22</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1552601.64</c:v>
+                  <c:v>126976.23</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6254,16 +7598,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>687382.03</c:v>
+                  <c:v>56250.74</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1044157.05</c:v>
+                  <c:v>90818.8</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1046676.37</c:v>
+                  <c:v>89422.22</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1552601.64</c:v>
+                  <c:v>126976.23</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7137,7 +8481,10 @@
         <c:spPr>
           <a:ln w="34925" cap="rnd">
             <a:solidFill>
-              <a:schemeClr val="lt1"/>
+              <a:schemeClr val="accent2">
+                <a:lumMod val="40000"/>
+                <a:lumOff val="60000"/>
+              </a:schemeClr>
             </a:solidFill>
             <a:round/>
           </a:ln>
@@ -7214,7 +8561,10 @@
         <c:spPr>
           <a:ln w="34925" cap="rnd">
             <a:solidFill>
-              <a:schemeClr val="lt1"/>
+              <a:schemeClr val="accent5">
+                <a:lumMod val="40000"/>
+                <a:lumOff val="60000"/>
+              </a:schemeClr>
             </a:solidFill>
             <a:round/>
           </a:ln>
@@ -7456,6 +8806,22 @@
               </c:spPr>
             </c:marker>
             <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:ln w="34925" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent2">
+                    <a:lumMod val="40000"/>
+                    <a:lumOff val="60000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:round/>
+              </a:ln>
+              <a:effectLst>
+                <a:outerShdw dist="25400" dir="2700000" algn="tl" rotWithShape="0">
+                  <a:schemeClr val="accent6"/>
+                </a:outerShdw>
+              </a:effectLst>
+            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000003-012B-4587-959B-9996804DB5A7}"/>
@@ -7481,6 +8847,22 @@
               </c:spPr>
             </c:marker>
             <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:ln w="34925" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent5">
+                    <a:lumMod val="40000"/>
+                    <a:lumOff val="60000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:round/>
+              </a:ln>
+              <a:effectLst>
+                <a:outerShdw dist="25400" dir="2700000" algn="tl" rotWithShape="0">
+                  <a:schemeClr val="accent6"/>
+                </a:outerShdw>
+              </a:effectLst>
+            </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000004-012B-4587-959B-9996804DB5A7}"/>
@@ -10341,7 +11723,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>851</c:v>
+                  <c:v>850</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -10499,22 +11881,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>4.2802E-2</c:v>
+                  <c:v>4.4330000000000001E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3.6144000000000003E-2</c:v>
+                  <c:v>3.5846999999999997E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.8516000000000001E-2</c:v>
+                  <c:v>1.6785999999999999E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.7103E-2</c:v>
+                  <c:v>1.4827999999999999E-2</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.70365100000000003</c:v>
+                  <c:v>0.71080200000000004</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.181784</c:v>
+                  <c:v>0.17740700000000001</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -15174,16 +16556,16 @@
       <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>88900</xdr:rowOff>
+      <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
       <xdr:colOff>596900</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>130172</xdr:rowOff>
+      <xdr:rowOff>136522</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-      <mc:Choice Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="5" name="month (Month)">
@@ -15206,7 +16588,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback xmlns="">
+      <mc:Fallback>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -15216,7 +16598,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="6807200" y="1746250"/>
+              <a:off x="6807200" y="1752600"/>
               <a:ext cx="1828800" cy="2619372"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -15955,654 +17337,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="Chantal Lee" refreshedDate="46142.821129976852" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{3728C892-97BF-4BD3-8C3A-33A379001046}">
-  <cacheSource type="external" connectionId="6"/>
-  <cacheFields count="5">
-    <cacheField name="[Month_by_Month_NY].[month].[month]" caption="month" numFmtId="0" hierarchy="16" level="1">
-      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2022-01-01T00:00:00" maxDate="2022-01-02T00:00:00" count="1">
-        <d v="2022-01-01T00:00:00"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="[Month_by_Month_NY].[month (Month)].[month (Month)]" caption="month (Month)" numFmtId="0" hierarchy="20" level="1">
-      <sharedItems count="3">
-        <s v="Jan"/>
-        <s v="Feb"/>
-        <s v="Mar"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="[Month_by_Month_NY].[month (Quarter)].[month (Quarter)]" caption="month (Quarter)" numFmtId="0" hierarchy="19" level="1">
-      <sharedItems count="4">
-        <s v="Qtr1"/>
-        <s v="Qtr2"/>
-        <s v="Qtr3"/>
-        <s v="Qtr4"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="[Month_by_Month_NY].[month (Year)].[month (Year)]" caption="month (Year)" numFmtId="0" hierarchy="18" level="1">
-      <sharedItems count="4">
-        <s v="2022"/>
-        <s v="2023"/>
-        <s v="2024"/>
-        <s v="2025"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="[Measures].[Sum of total_revenue 2]" caption="Sum of total_revenue 2" numFmtId="0" hierarchy="30" level="32767"/>
-  </cacheFields>
-  <cacheHierarchies count="36">
-    <cacheHierarchy uniqueName="[Category_Percentage_CT].[store_id]" caption="store_id" attribute="1" defaultMemberUniqueName="[Category_Percentage_CT].[store_id].[All]" allUniqueName="[Category_Percentage_CT].[store_id].[All]" dimensionUniqueName="[Category_Percentage_CT]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Category_Percentage_CT].[category]" caption="category" attribute="1" defaultMemberUniqueName="[Category_Percentage_CT].[category].[All]" allUniqueName="[Category_Percentage_CT].[category].[All]" dimensionUniqueName="[Category_Percentage_CT]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Category_Percentage_CT].[category_percentage]" caption="category_percentage" attribute="1" defaultMemberUniqueName="[Category_Percentage_CT].[category_percentage].[All]" allUniqueName="[Category_Percentage_CT].[category_percentage].[All]" dimensionUniqueName="[Category_Percentage_CT]" displayFolder="" count="0" memberValueDatatype="5" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Category_Percentage_NY].[store_id]" caption="store_id" attribute="1" defaultMemberUniqueName="[Category_Percentage_NY].[store_id].[All]" allUniqueName="[Category_Percentage_NY].[store_id].[All]" dimensionUniqueName="[Category_Percentage_NY]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Category_Percentage_NY].[category]" caption="category" attribute="1" defaultMemberUniqueName="[Category_Percentage_NY].[category].[All]" allUniqueName="[Category_Percentage_NY].[category].[All]" dimensionUniqueName="[Category_Percentage_NY]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Category_Percentage_NY].[category_percentage]" caption="category_percentage" attribute="1" defaultMemberUniqueName="[Category_Percentage_NY].[category_percentage].[All]" allUniqueName="[Category_Percentage_NY].[category_percentage].[All]" dimensionUniqueName="[Category_Percentage_NY]" displayFolder="" count="0" memberValueDatatype="5" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month].[Month]" caption="Month" attribute="1" time="1" defaultMemberUniqueName="[Month_by_Month].[Month].[All]" allUniqueName="[Month_by_Month].[Month].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="0" memberValueDatatype="7" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month].[Total_Revenue]" caption="Total_Revenue" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Total_Revenue].[All]" allUniqueName="[Month_by_Month].[Total_Revenue].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="0" memberValueDatatype="5" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month].[Month (Year)]" caption="Month (Year)" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Month (Year)].[All]" allUniqueName="[Month_by_Month].[Month (Year)].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month].[Month (Quarter)]" caption="Month (Quarter)" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Month (Quarter)].[All]" allUniqueName="[Month_by_Month].[Month (Quarter)].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month].[Month (Month)]" caption="Month (Month)" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Month (Month)].[All]" allUniqueName="[Month_by_Month].[Month (Month)].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month]" caption="month" attribute="1" time="1" defaultMemberUniqueName="[Month_by_Month_CT].[month].[All]" allUniqueName="[Month_by_Month_CT].[month].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="0" memberValueDatatype="7" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_CT].[total_revenue]" caption="total_revenue" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[total_revenue].[All]" allUniqueName="[Month_by_Month_CT].[total_revenue].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="0" memberValueDatatype="5" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month (Year)]" caption="month (Year)" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[month (Year)].[All]" allUniqueName="[Month_by_Month_CT].[month (Year)].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month (Quarter)]" caption="month (Quarter)" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[month (Quarter)].[All]" allUniqueName="[Month_by_Month_CT].[month (Quarter)].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month (Month)]" caption="month (Month)" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[month (Month)].[All]" allUniqueName="[Month_by_Month_CT].[month (Month)].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month]" caption="month" attribute="1" time="1" defaultMemberUniqueName="[Month_by_Month_NY].[month].[All]" allUniqueName="[Month_by_Month_NY].[month].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="2" memberValueDatatype="7" unbalanced="0">
-      <fieldsUsage count="2">
-        <fieldUsage x="-1"/>
-        <fieldUsage x="0"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Month_by_Month_NY].[total_revenue]" caption="total_revenue" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[total_revenue].[All]" allUniqueName="[Month_by_Month_NY].[total_revenue].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="0" memberValueDatatype="5" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month (Year)]" caption="month (Year)" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[month (Year)].[All]" allUniqueName="[Month_by_Month_NY].[month (Year)].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0">
-      <fieldsUsage count="2">
-        <fieldUsage x="-1"/>
-        <fieldUsage x="3"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month (Quarter)]" caption="month (Quarter)" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[month (Quarter)].[All]" allUniqueName="[Month_by_Month_NY].[month (Quarter)].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0">
-      <fieldsUsage count="2">
-        <fieldUsage x="-1"/>
-        <fieldUsage x="2"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month (Month)]" caption="month (Month)" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[month (Month)].[All]" allUniqueName="[Month_by_Month_NY].[month (Month)].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0">
-      <fieldsUsage count="2">
-        <fieldUsage x="-1"/>
-        <fieldUsage x="1"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Month_by_Month].[Month (Month Index)]" caption="Month (Month Index)" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Month (Month Index)].[All]" allUniqueName="[Month_by_Month].[Month (Month Index)].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month (Month Index)]" caption="month (Month Index)" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[month (Month Index)].[All]" allUniqueName="[Month_by_Month_CT].[month (Month Index)].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month (Month Index)]" caption="month (Month Index)" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[month (Month Index)].[All]" allUniqueName="[Month_by_Month_NY].[month (Month Index)].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[__XL_Count Month_by_Month_NY]" caption="__XL_Count Month_by_Month_NY" measure="1" displayFolder="" measureGroup="Month_by_Month_NY" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[__XL_Count Month_by_Month_CT]" caption="__XL_Count Month_by_Month_CT" measure="1" displayFolder="" measureGroup="Month_by_Month_CT" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[__XL_Count Month_by_Month]" caption="__XL_Count Month_by_Month" measure="1" displayFolder="" measureGroup="Month_by_Month" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[__XL_Count Category_Percentage_CT]" caption="__XL_Count Category_Percentage_CT" measure="1" displayFolder="" measureGroup="Category_Percentage_CT" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[__XL_Count Category_Percentage_NY]" caption="__XL_Count Category_Percentage_NY" measure="1" displayFolder="" measureGroup="Category_Percentage_NY" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[__No measures defined]" caption="__No measures defined" measure="1" displayFolder="" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[Sum of total_revenue 2]" caption="Sum of total_revenue 2" measure="1" displayFolder="" measureGroup="Month_by_Month_NY" count="0" oneField="1" hidden="1">
-      <fieldsUsage count="1">
-        <fieldUsage x="4"/>
-      </fieldsUsage>
-      <extLst>
-        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
-          <x15:cacheHierarchy aggregatedColumn="17"/>
-        </ext>
-      </extLst>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Measures].[Sum of total_revenue]" caption="Sum of total_revenue" measure="1" displayFolder="" measureGroup="Month_by_Month_CT" count="0" hidden="1">
-      <extLst>
-        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
-          <x15:cacheHierarchy aggregatedColumn="12"/>
-        </ext>
-      </extLst>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Measures].[Sum of Total_Revenue 3]" caption="Sum of Total_Revenue 3" measure="1" displayFolder="" measureGroup="Month_by_Month" count="0" hidden="1">
-      <extLst>
-        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
-          <x15:cacheHierarchy aggregatedColumn="7"/>
-        </ext>
-      </extLst>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Measures].[Sum of category_percentage]" caption="Sum of category_percentage" measure="1" displayFolder="" measureGroup="Category_Percentage_CT" count="0" hidden="1">
-      <extLst>
-        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
-          <x15:cacheHierarchy aggregatedColumn="2"/>
-        </ext>
-      </extLst>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Measures].[Sum of store_id]" caption="Sum of store_id" measure="1" displayFolder="" measureGroup="Category_Percentage_CT" count="0" hidden="1">
-      <extLst>
-        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
-          <x15:cacheHierarchy aggregatedColumn="0"/>
-        </ext>
-      </extLst>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Measures].[Sum of category_percentage 2]" caption="Sum of category_percentage 2" measure="1" displayFolder="" measureGroup="Category_Percentage_NY" count="0" hidden="1">
-      <extLst>
-        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
-          <x15:cacheHierarchy aggregatedColumn="5"/>
-        </ext>
-      </extLst>
-    </cacheHierarchy>
-  </cacheHierarchies>
-  <kpis count="0"/>
-  <dimensions count="6">
-    <dimension name="Category_Percentage_CT" uniqueName="[Category_Percentage_CT]" caption="Category_Percentage_CT"/>
-    <dimension name="Category_Percentage_NY" uniqueName="[Category_Percentage_NY]" caption="Category_Percentage_NY"/>
-    <dimension measure="1" name="Measures" uniqueName="[Measures]" caption="Measures"/>
-    <dimension name="Month_by_Month" uniqueName="[Month_by_Month]" caption="Month_by_Month"/>
-    <dimension name="Month_by_Month_CT" uniqueName="[Month_by_Month_CT]" caption="Month_by_Month_CT"/>
-    <dimension name="Month_by_Month_NY" uniqueName="[Month_by_Month_NY]" caption="Month_by_Month_NY"/>
-  </dimensions>
-  <measureGroups count="5">
-    <measureGroup name="Category_Percentage_CT" caption="Category_Percentage_CT"/>
-    <measureGroup name="Category_Percentage_NY" caption="Category_Percentage_NY"/>
-    <measureGroup name="Month_by_Month" caption="Month_by_Month"/>
-    <measureGroup name="Month_by_Month_CT" caption="Month_by_Month_CT"/>
-    <measureGroup name="Month_by_Month_NY" caption="Month_by_Month_NY"/>
-  </measureGroups>
-  <maps count="5">
-    <map measureGroup="0" dimension="0"/>
-    <map measureGroup="1" dimension="1"/>
-    <map measureGroup="2" dimension="3"/>
-    <map measureGroup="3" dimension="4"/>
-    <map measureGroup="4" dimension="5"/>
-  </maps>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition supportSubqueryNonVisual="1" supportSubqueryCalcMem="1" supportAddCalcMems="1"/>
-    </ext>
-  </extLst>
-</pivotCacheDefinition>
-</file>
-
-<file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="Chantal Lee" refreshedDate="46142.878276388888" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{B0A6EEAC-EAE3-4C7C-BC5A-70188D13667D}">
-  <cacheSource type="external" connectionId="6"/>
-  <cacheFields count="5">
-    <cacheField name="[Month_by_Month_CT].[month].[month]" caption="month" numFmtId="0" hierarchy="11" level="1">
-      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2024-09-01T00:00:00" maxDate="2024-09-02T00:00:00" count="1">
-        <d v="2024-09-01T00:00:00"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="[Month_by_Month_CT].[month (Month)].[month (Month)]" caption="month (Month)" numFmtId="0" hierarchy="15" level="1">
-      <sharedItems count="1">
-        <s v="Sep"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="[Month_by_Month_CT].[month (Quarter)].[month (Quarter)]" caption="month (Quarter)" numFmtId="0" hierarchy="14" level="1">
-      <sharedItems count="1">
-        <s v="Qtr3"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="[Month_by_Month_CT].[month (Year)].[month (Year)]" caption="month (Year)" numFmtId="0" hierarchy="13" level="1">
-      <sharedItems count="4">
-        <s v="2022"/>
-        <s v="2023"/>
-        <s v="2024"/>
-        <s v="2025"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="[Measures].[Sum of total_revenue]" caption="Sum of total_revenue" numFmtId="0" hierarchy="31" level="32767"/>
-  </cacheFields>
-  <cacheHierarchies count="36">
-    <cacheHierarchy uniqueName="[Category_Percentage_CT].[store_id]" caption="store_id" attribute="1" defaultMemberUniqueName="[Category_Percentage_CT].[store_id].[All]" allUniqueName="[Category_Percentage_CT].[store_id].[All]" dimensionUniqueName="[Category_Percentage_CT]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Category_Percentage_CT].[category]" caption="category" attribute="1" defaultMemberUniqueName="[Category_Percentage_CT].[category].[All]" allUniqueName="[Category_Percentage_CT].[category].[All]" dimensionUniqueName="[Category_Percentage_CT]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Category_Percentage_CT].[category_percentage]" caption="category_percentage" attribute="1" defaultMemberUniqueName="[Category_Percentage_CT].[category_percentage].[All]" allUniqueName="[Category_Percentage_CT].[category_percentage].[All]" dimensionUniqueName="[Category_Percentage_CT]" displayFolder="" count="0" memberValueDatatype="5" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Category_Percentage_NY].[store_id]" caption="store_id" attribute="1" defaultMemberUniqueName="[Category_Percentage_NY].[store_id].[All]" allUniqueName="[Category_Percentage_NY].[store_id].[All]" dimensionUniqueName="[Category_Percentage_NY]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Category_Percentage_NY].[category]" caption="category" attribute="1" defaultMemberUniqueName="[Category_Percentage_NY].[category].[All]" allUniqueName="[Category_Percentage_NY].[category].[All]" dimensionUniqueName="[Category_Percentage_NY]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Category_Percentage_NY].[category_percentage]" caption="category_percentage" attribute="1" defaultMemberUniqueName="[Category_Percentage_NY].[category_percentage].[All]" allUniqueName="[Category_Percentage_NY].[category_percentage].[All]" dimensionUniqueName="[Category_Percentage_NY]" displayFolder="" count="0" memberValueDatatype="5" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month].[Month]" caption="Month" attribute="1" time="1" defaultMemberUniqueName="[Month_by_Month].[Month].[All]" allUniqueName="[Month_by_Month].[Month].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="0" memberValueDatatype="7" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month].[Total_Revenue]" caption="Total_Revenue" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Total_Revenue].[All]" allUniqueName="[Month_by_Month].[Total_Revenue].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="0" memberValueDatatype="5" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month].[Month (Year)]" caption="Month (Year)" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Month (Year)].[All]" allUniqueName="[Month_by_Month].[Month (Year)].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month].[Month (Quarter)]" caption="Month (Quarter)" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Month (Quarter)].[All]" allUniqueName="[Month_by_Month].[Month (Quarter)].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month].[Month (Month)]" caption="Month (Month)" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Month (Month)].[All]" allUniqueName="[Month_by_Month].[Month (Month)].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month]" caption="month" attribute="1" time="1" defaultMemberUniqueName="[Month_by_Month_CT].[month].[All]" allUniqueName="[Month_by_Month_CT].[month].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="2" memberValueDatatype="7" unbalanced="0">
-      <fieldsUsage count="2">
-        <fieldUsage x="-1"/>
-        <fieldUsage x="0"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Month_by_Month_CT].[total_revenue]" caption="total_revenue" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[total_revenue].[All]" allUniqueName="[Month_by_Month_CT].[total_revenue].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="0" memberValueDatatype="5" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month (Year)]" caption="month (Year)" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[month (Year)].[All]" allUniqueName="[Month_by_Month_CT].[month (Year)].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0">
-      <fieldsUsage count="2">
-        <fieldUsage x="-1"/>
-        <fieldUsage x="3"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month (Quarter)]" caption="month (Quarter)" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[month (Quarter)].[All]" allUniqueName="[Month_by_Month_CT].[month (Quarter)].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0">
-      <fieldsUsage count="2">
-        <fieldUsage x="-1"/>
-        <fieldUsage x="2"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month (Month)]" caption="month (Month)" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[month (Month)].[All]" allUniqueName="[Month_by_Month_CT].[month (Month)].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0">
-      <fieldsUsage count="2">
-        <fieldUsage x="-1"/>
-        <fieldUsage x="1"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month]" caption="month" attribute="1" time="1" defaultMemberUniqueName="[Month_by_Month_NY].[month].[All]" allUniqueName="[Month_by_Month_NY].[month].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="0" memberValueDatatype="7" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_NY].[total_revenue]" caption="total_revenue" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[total_revenue].[All]" allUniqueName="[Month_by_Month_NY].[total_revenue].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="0" memberValueDatatype="5" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month (Year)]" caption="month (Year)" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[month (Year)].[All]" allUniqueName="[Month_by_Month_NY].[month (Year)].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month (Quarter)]" caption="month (Quarter)" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[month (Quarter)].[All]" allUniqueName="[Month_by_Month_NY].[month (Quarter)].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month (Month)]" caption="month (Month)" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[month (Month)].[All]" allUniqueName="[Month_by_Month_NY].[month (Month)].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month].[Month (Month Index)]" caption="Month (Month Index)" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Month (Month Index)].[All]" allUniqueName="[Month_by_Month].[Month (Month Index)].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month (Month Index)]" caption="month (Month Index)" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[month (Month Index)].[All]" allUniqueName="[Month_by_Month_CT].[month (Month Index)].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month (Month Index)]" caption="month (Month Index)" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[month (Month Index)].[All]" allUniqueName="[Month_by_Month_NY].[month (Month Index)].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[__XL_Count Month_by_Month_NY]" caption="__XL_Count Month_by_Month_NY" measure="1" displayFolder="" measureGroup="Month_by_Month_NY" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[__XL_Count Month_by_Month_CT]" caption="__XL_Count Month_by_Month_CT" measure="1" displayFolder="" measureGroup="Month_by_Month_CT" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[__XL_Count Month_by_Month]" caption="__XL_Count Month_by_Month" measure="1" displayFolder="" measureGroup="Month_by_Month" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[__XL_Count Category_Percentage_CT]" caption="__XL_Count Category_Percentage_CT" measure="1" displayFolder="" measureGroup="Category_Percentage_CT" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[__XL_Count Category_Percentage_NY]" caption="__XL_Count Category_Percentage_NY" measure="1" displayFolder="" measureGroup="Category_Percentage_NY" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[__No measures defined]" caption="__No measures defined" measure="1" displayFolder="" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[Sum of total_revenue 2]" caption="Sum of total_revenue 2" measure="1" displayFolder="" measureGroup="Month_by_Month_NY" count="0" hidden="1">
-      <extLst>
-        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
-          <x15:cacheHierarchy aggregatedColumn="17"/>
-        </ext>
-      </extLst>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Measures].[Sum of total_revenue]" caption="Sum of total_revenue" measure="1" displayFolder="" measureGroup="Month_by_Month_CT" count="0" oneField="1" hidden="1">
-      <fieldsUsage count="1">
-        <fieldUsage x="4"/>
-      </fieldsUsage>
-      <extLst>
-        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
-          <x15:cacheHierarchy aggregatedColumn="12"/>
-        </ext>
-      </extLst>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Measures].[Sum of Total_Revenue 3]" caption="Sum of Total_Revenue 3" measure="1" displayFolder="" measureGroup="Month_by_Month" count="0" hidden="1">
-      <extLst>
-        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
-          <x15:cacheHierarchy aggregatedColumn="7"/>
-        </ext>
-      </extLst>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Measures].[Sum of category_percentage]" caption="Sum of category_percentage" measure="1" displayFolder="" measureGroup="Category_Percentage_CT" count="0" hidden="1">
-      <extLst>
-        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
-          <x15:cacheHierarchy aggregatedColumn="2"/>
-        </ext>
-      </extLst>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Measures].[Sum of store_id]" caption="Sum of store_id" measure="1" displayFolder="" measureGroup="Category_Percentage_CT" count="0" hidden="1">
-      <extLst>
-        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
-          <x15:cacheHierarchy aggregatedColumn="0"/>
-        </ext>
-      </extLst>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Measures].[Sum of category_percentage 2]" caption="Sum of category_percentage 2" measure="1" displayFolder="" measureGroup="Category_Percentage_NY" count="0" hidden="1">
-      <extLst>
-        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
-          <x15:cacheHierarchy aggregatedColumn="5"/>
-        </ext>
-      </extLst>
-    </cacheHierarchy>
-  </cacheHierarchies>
-  <kpis count="0"/>
-  <dimensions count="6">
-    <dimension name="Category_Percentage_CT" uniqueName="[Category_Percentage_CT]" caption="Category_Percentage_CT"/>
-    <dimension name="Category_Percentage_NY" uniqueName="[Category_Percentage_NY]" caption="Category_Percentage_NY"/>
-    <dimension measure="1" name="Measures" uniqueName="[Measures]" caption="Measures"/>
-    <dimension name="Month_by_Month" uniqueName="[Month_by_Month]" caption="Month_by_Month"/>
-    <dimension name="Month_by_Month_CT" uniqueName="[Month_by_Month_CT]" caption="Month_by_Month_CT"/>
-    <dimension name="Month_by_Month_NY" uniqueName="[Month_by_Month_NY]" caption="Month_by_Month_NY"/>
-  </dimensions>
-  <measureGroups count="5">
-    <measureGroup name="Category_Percentage_CT" caption="Category_Percentage_CT"/>
-    <measureGroup name="Category_Percentage_NY" caption="Category_Percentage_NY"/>
-    <measureGroup name="Month_by_Month" caption="Month_by_Month"/>
-    <measureGroup name="Month_by_Month_CT" caption="Month_by_Month_CT"/>
-    <measureGroup name="Month_by_Month_NY" caption="Month_by_Month_NY"/>
-  </measureGroups>
-  <maps count="5">
-    <map measureGroup="0" dimension="0"/>
-    <map measureGroup="1" dimension="1"/>
-    <map measureGroup="2" dimension="3"/>
-    <map measureGroup="3" dimension="4"/>
-    <map measureGroup="4" dimension="5"/>
-  </maps>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition supportSubqueryNonVisual="1" supportSubqueryCalcMem="1" supportAddCalcMems="1"/>
-    </ext>
-  </extLst>
-</pivotCacheDefinition>
-</file>
-
-<file path=xl/pivotCache/pivotCacheDefinition3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="Chantal Lee" refreshedDate="46142.902477777781" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{9CCA98CC-7441-4E2D-BA36-575067284E5B}">
-  <cacheSource type="external" connectionId="6"/>
-  <cacheFields count="3">
-    <cacheField name="[Category_Percentage_CT].[category].[category]" caption="category" numFmtId="0" hierarchy="1" level="1">
-      <sharedItems count="6">
-        <s v="Apparel and Merchandise"/>
-        <s v="Art Supplies"/>
-        <s v="Books (General)"/>
-        <s v="Stationery and Supplies"/>
-        <s v="Technology &amp; Accessories"/>
-        <s v="Textbooks"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="[Measures].[Sum of category_percentage]" caption="Sum of category_percentage" numFmtId="0" hierarchy="33" level="32767"/>
-    <cacheField name="[Category_Percentage_CT].[store_id].[store_id]" caption="store_id" numFmtId="0" level="1">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="865" maxValue="872" count="8">
-        <n v="870"/>
-        <n v="871" u="1"/>
-        <n v="865" u="1"/>
-        <n v="866" u="1"/>
-        <n v="867" u="1"/>
-        <n v="868" u="1"/>
-        <n v="869" u="1"/>
-        <n v="872" u="1"/>
-      </sharedItems>
-      <extLst>
-        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{4F2E5C28-24EA-4eb8-9CBF-B6C8F9C3D259}">
-          <x15:cachedUniqueNames>
-            <x15:cachedUniqueName index="0" name="[Category_Percentage_CT].[store_id].&amp;[870]"/>
-            <x15:cachedUniqueName index="1" name="[Category_Percentage_CT].[store_id].&amp;[871]"/>
-            <x15:cachedUniqueName index="2" name="[Category_Percentage_CT].[store_id].&amp;[865]"/>
-            <x15:cachedUniqueName index="3" name="[Category_Percentage_CT].[store_id].&amp;[866]"/>
-            <x15:cachedUniqueName index="4" name="[Category_Percentage_CT].[store_id].&amp;[867]"/>
-            <x15:cachedUniqueName index="5" name="[Category_Percentage_CT].[store_id].&amp;[868]"/>
-            <x15:cachedUniqueName index="6" name="[Category_Percentage_CT].[store_id].&amp;[869]"/>
-            <x15:cachedUniqueName index="7" name="[Category_Percentage_CT].[store_id].&amp;[872]"/>
-          </x15:cachedUniqueNames>
-        </ext>
-      </extLst>
-    </cacheField>
-  </cacheFields>
-  <cacheHierarchies count="36">
-    <cacheHierarchy uniqueName="[Category_Percentage_CT].[store_id]" caption="store_id" attribute="1" defaultMemberUniqueName="[Category_Percentage_CT].[store_id].[All]" allUniqueName="[Category_Percentage_CT].[store_id].[All]" dimensionUniqueName="[Category_Percentage_CT]" displayFolder="" count="2" memberValueDatatype="20" unbalanced="0">
-      <fieldsUsage count="2">
-        <fieldUsage x="-1"/>
-        <fieldUsage x="2"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Category_Percentage_CT].[category]" caption="category" attribute="1" defaultMemberUniqueName="[Category_Percentage_CT].[category].[All]" allUniqueName="[Category_Percentage_CT].[category].[All]" dimensionUniqueName="[Category_Percentage_CT]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0">
-      <fieldsUsage count="2">
-        <fieldUsage x="-1"/>
-        <fieldUsage x="0"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Category_Percentage_CT].[category_percentage]" caption="category_percentage" attribute="1" defaultMemberUniqueName="[Category_Percentage_CT].[category_percentage].[All]" allUniqueName="[Category_Percentage_CT].[category_percentage].[All]" dimensionUniqueName="[Category_Percentage_CT]" displayFolder="" count="2" memberValueDatatype="5" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Category_Percentage_NY].[store_id]" caption="store_id" attribute="1" defaultMemberUniqueName="[Category_Percentage_NY].[store_id].[All]" allUniqueName="[Category_Percentage_NY].[store_id].[All]" dimensionUniqueName="[Category_Percentage_NY]" displayFolder="" count="2" memberValueDatatype="20" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Category_Percentage_NY].[category]" caption="category" attribute="1" defaultMemberUniqueName="[Category_Percentage_NY].[category].[All]" allUniqueName="[Category_Percentage_NY].[category].[All]" dimensionUniqueName="[Category_Percentage_NY]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Category_Percentage_NY].[category_percentage]" caption="category_percentage" attribute="1" defaultMemberUniqueName="[Category_Percentage_NY].[category_percentage].[All]" allUniqueName="[Category_Percentage_NY].[category_percentage].[All]" dimensionUniqueName="[Category_Percentage_NY]" displayFolder="" count="2" memberValueDatatype="5" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month].[Month]" caption="Month" attribute="1" time="1" defaultMemberUniqueName="[Month_by_Month].[Month].[All]" allUniqueName="[Month_by_Month].[Month].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="2" memberValueDatatype="7" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month].[Total_Revenue]" caption="Total_Revenue" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Total_Revenue].[All]" allUniqueName="[Month_by_Month].[Total_Revenue].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="2" memberValueDatatype="5" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month].[Month (Year)]" caption="Month (Year)" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Month (Year)].[All]" allUniqueName="[Month_by_Month].[Month (Year)].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month].[Month (Quarter)]" caption="Month (Quarter)" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Month (Quarter)].[All]" allUniqueName="[Month_by_Month].[Month (Quarter)].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month].[Month (Month)]" caption="Month (Month)" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Month (Month)].[All]" allUniqueName="[Month_by_Month].[Month (Month)].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month]" caption="month" attribute="1" time="1" defaultMemberUniqueName="[Month_by_Month_CT].[month].[All]" allUniqueName="[Month_by_Month_CT].[month].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="2" memberValueDatatype="7" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_CT].[total_revenue]" caption="total_revenue" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[total_revenue].[All]" allUniqueName="[Month_by_Month_CT].[total_revenue].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="2" memberValueDatatype="5" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month (Year)]" caption="month (Year)" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[month (Year)].[All]" allUniqueName="[Month_by_Month_CT].[month (Year)].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month (Quarter)]" caption="month (Quarter)" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[month (Quarter)].[All]" allUniqueName="[Month_by_Month_CT].[month (Quarter)].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month (Month)]" caption="month (Month)" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[month (Month)].[All]" allUniqueName="[Month_by_Month_CT].[month (Month)].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month]" caption="month" attribute="1" time="1" defaultMemberUniqueName="[Month_by_Month_NY].[month].[All]" allUniqueName="[Month_by_Month_NY].[month].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="2" memberValueDatatype="7" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_NY].[total_revenue]" caption="total_revenue" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[total_revenue].[All]" allUniqueName="[Month_by_Month_NY].[total_revenue].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="2" memberValueDatatype="5" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month (Year)]" caption="month (Year)" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[month (Year)].[All]" allUniqueName="[Month_by_Month_NY].[month (Year)].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month (Quarter)]" caption="month (Quarter)" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[month (Quarter)].[All]" allUniqueName="[Month_by_Month_NY].[month (Quarter)].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month (Month)]" caption="month (Month)" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[month (Month)].[All]" allUniqueName="[Month_by_Month_NY].[month (Month)].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month].[Month (Month Index)]" caption="Month (Month Index)" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Month (Month Index)].[All]" allUniqueName="[Month_by_Month].[Month (Month Index)].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="2" memberValueDatatype="20" unbalanced="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month (Month Index)]" caption="month (Month Index)" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[month (Month Index)].[All]" allUniqueName="[Month_by_Month_CT].[month (Month Index)].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="2" memberValueDatatype="20" unbalanced="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month (Month Index)]" caption="month (Month Index)" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[month (Month Index)].[All]" allUniqueName="[Month_by_Month_NY].[month (Month Index)].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="2" memberValueDatatype="20" unbalanced="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[__XL_Count Month_by_Month_NY]" caption="__XL_Count Month_by_Month_NY" measure="1" displayFolder="" measureGroup="Month_by_Month_NY" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[__XL_Count Month_by_Month_CT]" caption="__XL_Count Month_by_Month_CT" measure="1" displayFolder="" measureGroup="Month_by_Month_CT" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[__XL_Count Month_by_Month]" caption="__XL_Count Month_by_Month" measure="1" displayFolder="" measureGroup="Month_by_Month" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[__XL_Count Category_Percentage_CT]" caption="__XL_Count Category_Percentage_CT" measure="1" displayFolder="" measureGroup="Category_Percentage_CT" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[__XL_Count Category_Percentage_NY]" caption="__XL_Count Category_Percentage_NY" measure="1" displayFolder="" measureGroup="Category_Percentage_NY" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[__No measures defined]" caption="__No measures defined" measure="1" displayFolder="" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[Sum of total_revenue 2]" caption="Sum of total_revenue 2" measure="1" displayFolder="" measureGroup="Month_by_Month_NY" count="0" hidden="1">
-      <extLst>
-        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
-          <x15:cacheHierarchy aggregatedColumn="17"/>
-        </ext>
-      </extLst>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Measures].[Sum of total_revenue]" caption="Sum of total_revenue" measure="1" displayFolder="" measureGroup="Month_by_Month_CT" count="0" hidden="1">
-      <extLst>
-        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
-          <x15:cacheHierarchy aggregatedColumn="12"/>
-        </ext>
-      </extLst>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Measures].[Sum of Total_Revenue 3]" caption="Sum of Total_Revenue 3" measure="1" displayFolder="" measureGroup="Month_by_Month" count="0" hidden="1">
-      <extLst>
-        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
-          <x15:cacheHierarchy aggregatedColumn="7"/>
-        </ext>
-      </extLst>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Measures].[Sum of category_percentage]" caption="Sum of category_percentage" measure="1" displayFolder="" measureGroup="Category_Percentage_CT" count="0" oneField="1" hidden="1">
-      <fieldsUsage count="1">
-        <fieldUsage x="1"/>
-      </fieldsUsage>
-      <extLst>
-        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
-          <x15:cacheHierarchy aggregatedColumn="2"/>
-        </ext>
-      </extLst>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Measures].[Sum of store_id]" caption="Sum of store_id" measure="1" displayFolder="" measureGroup="Category_Percentage_CT" count="0" hidden="1">
-      <extLst>
-        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
-          <x15:cacheHierarchy aggregatedColumn="0"/>
-        </ext>
-      </extLst>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Measures].[Sum of category_percentage 2]" caption="Sum of category_percentage 2" measure="1" displayFolder="" measureGroup="Category_Percentage_NY" count="0" hidden="1">
-      <extLst>
-        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
-          <x15:cacheHierarchy aggregatedColumn="5"/>
-        </ext>
-      </extLst>
-    </cacheHierarchy>
-  </cacheHierarchies>
-  <kpis count="0"/>
-  <dimensions count="6">
-    <dimension name="Category_Percentage_CT" uniqueName="[Category_Percentage_CT]" caption="Category_Percentage_CT"/>
-    <dimension name="Category_Percentage_NY" uniqueName="[Category_Percentage_NY]" caption="Category_Percentage_NY"/>
-    <dimension measure="1" name="Measures" uniqueName="[Measures]" caption="Measures"/>
-    <dimension name="Month_by_Month" uniqueName="[Month_by_Month]" caption="Month_by_Month"/>
-    <dimension name="Month_by_Month_CT" uniqueName="[Month_by_Month_CT]" caption="Month_by_Month_CT"/>
-    <dimension name="Month_by_Month_NY" uniqueName="[Month_by_Month_NY]" caption="Month_by_Month_NY"/>
-  </dimensions>
-  <measureGroups count="5">
-    <measureGroup name="Category_Percentage_CT" caption="Category_Percentage_CT"/>
-    <measureGroup name="Category_Percentage_NY" caption="Category_Percentage_NY"/>
-    <measureGroup name="Month_by_Month" caption="Month_by_Month"/>
-    <measureGroup name="Month_by_Month_CT" caption="Month_by_Month_CT"/>
-    <measureGroup name="Month_by_Month_NY" caption="Month_by_Month_NY"/>
-  </measureGroups>
-  <maps count="5">
-    <map measureGroup="0" dimension="0"/>
-    <map measureGroup="1" dimension="1"/>
-    <map measureGroup="2" dimension="3"/>
-    <map measureGroup="3" dimension="4"/>
-    <map measureGroup="4" dimension="5"/>
-  </maps>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition supportSubqueryNonVisual="1" supportSubqueryCalcMem="1" supportAddCalcMems="1"/>
-    </ext>
-  </extLst>
-</pivotCacheDefinition>
-</file>
-
-<file path=xl/pivotCache/pivotCacheDefinition4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="Chantal Lee" refreshedDate="46142.902734027775" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{0CC7DB6F-F048-4B9F-B9D9-C2E5CD0C5F47}">
-  <cacheSource type="external" connectionId="6"/>
-  <cacheFields count="3">
-    <cacheField name="[Category_Percentage_NY].[store_id].[store_id]" caption="store_id" numFmtId="0" hierarchy="3" level="1">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="840" maxValue="851" count="12">
-        <n v="851"/>
-        <n v="850" u="1"/>
-        <n v="846" u="1"/>
-        <n v="847" u="1"/>
-        <n v="840" u="1"/>
-        <n v="841" u="1"/>
-        <n v="842" u="1"/>
-        <n v="843" u="1"/>
-        <n v="844" u="1"/>
-        <n v="845" u="1"/>
-        <n v="848" u="1"/>
-        <n v="849" u="1"/>
-      </sharedItems>
-      <extLst>
-        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{4F2E5C28-24EA-4eb8-9CBF-B6C8F9C3D259}">
-          <x15:cachedUniqueNames>
-            <x15:cachedUniqueName index="0" name="[Category_Percentage_NY].[store_id].&amp;[851]"/>
-            <x15:cachedUniqueName index="1" name="[Category_Percentage_NY].[store_id].&amp;[850]"/>
-            <x15:cachedUniqueName index="2" name="[Category_Percentage_NY].[store_id].&amp;[846]"/>
-            <x15:cachedUniqueName index="3" name="[Category_Percentage_NY].[store_id].&amp;[847]"/>
-            <x15:cachedUniqueName index="4" name="[Category_Percentage_NY].[store_id].&amp;[840]"/>
-            <x15:cachedUniqueName index="5" name="[Category_Percentage_NY].[store_id].&amp;[841]"/>
-            <x15:cachedUniqueName index="6" name="[Category_Percentage_NY].[store_id].&amp;[842]"/>
-            <x15:cachedUniqueName index="7" name="[Category_Percentage_NY].[store_id].&amp;[843]"/>
-            <x15:cachedUniqueName index="8" name="[Category_Percentage_NY].[store_id].&amp;[844]"/>
-            <x15:cachedUniqueName index="9" name="[Category_Percentage_NY].[store_id].&amp;[845]"/>
-            <x15:cachedUniqueName index="10" name="[Category_Percentage_NY].[store_id].&amp;[848]"/>
-            <x15:cachedUniqueName index="11" name="[Category_Percentage_NY].[store_id].&amp;[849]"/>
-          </x15:cachedUniqueNames>
-        </ext>
-      </extLst>
-    </cacheField>
-    <cacheField name="[Measures].[Sum of category_percentage 2]" caption="Sum of category_percentage 2" numFmtId="0" hierarchy="35" level="32767"/>
-    <cacheField name="[Category_Percentage_NY].[category].[category]" caption="category" numFmtId="0" hierarchy="4" level="1">
-      <sharedItems count="6">
-        <s v="Apparel and Merchandise"/>
-        <s v="Art Supplies"/>
-        <s v="Books (General)"/>
-        <s v="Stationery and Supplies"/>
-        <s v="Technology &amp; Accessories"/>
-        <s v="Textbooks"/>
-      </sharedItems>
-    </cacheField>
-  </cacheFields>
-  <cacheHierarchies count="36">
-    <cacheHierarchy uniqueName="[Category_Percentage_CT].[store_id]" caption="store_id" attribute="1" defaultMemberUniqueName="[Category_Percentage_CT].[store_id].[All]" allUniqueName="[Category_Percentage_CT].[store_id].[All]" dimensionUniqueName="[Category_Percentage_CT]" displayFolder="" count="2" memberValueDatatype="20" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Category_Percentage_CT].[category]" caption="category" attribute="1" defaultMemberUniqueName="[Category_Percentage_CT].[category].[All]" allUniqueName="[Category_Percentage_CT].[category].[All]" dimensionUniqueName="[Category_Percentage_CT]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Category_Percentage_CT].[category_percentage]" caption="category_percentage" attribute="1" defaultMemberUniqueName="[Category_Percentage_CT].[category_percentage].[All]" allUniqueName="[Category_Percentage_CT].[category_percentage].[All]" dimensionUniqueName="[Category_Percentage_CT]" displayFolder="" count="2" memberValueDatatype="5" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Category_Percentage_NY].[store_id]" caption="store_id" attribute="1" defaultMemberUniqueName="[Category_Percentage_NY].[store_id].[All]" allUniqueName="[Category_Percentage_NY].[store_id].[All]" dimensionUniqueName="[Category_Percentage_NY]" displayFolder="" count="2" memberValueDatatype="20" unbalanced="0">
-      <fieldsUsage count="2">
-        <fieldUsage x="-1"/>
-        <fieldUsage x="0"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Category_Percentage_NY].[category]" caption="category" attribute="1" defaultMemberUniqueName="[Category_Percentage_NY].[category].[All]" allUniqueName="[Category_Percentage_NY].[category].[All]" dimensionUniqueName="[Category_Percentage_NY]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0">
-      <fieldsUsage count="2">
-        <fieldUsage x="-1"/>
-        <fieldUsage x="2"/>
-      </fieldsUsage>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Category_Percentage_NY].[category_percentage]" caption="category_percentage" attribute="1" defaultMemberUniqueName="[Category_Percentage_NY].[category_percentage].[All]" allUniqueName="[Category_Percentage_NY].[category_percentage].[All]" dimensionUniqueName="[Category_Percentage_NY]" displayFolder="" count="2" memberValueDatatype="5" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month].[Month]" caption="Month" attribute="1" time="1" defaultMemberUniqueName="[Month_by_Month].[Month].[All]" allUniqueName="[Month_by_Month].[Month].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="2" memberValueDatatype="7" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month].[Total_Revenue]" caption="Total_Revenue" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Total_Revenue].[All]" allUniqueName="[Month_by_Month].[Total_Revenue].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="2" memberValueDatatype="5" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month].[Month (Year)]" caption="Month (Year)" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Month (Year)].[All]" allUniqueName="[Month_by_Month].[Month (Year)].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month].[Month (Quarter)]" caption="Month (Quarter)" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Month (Quarter)].[All]" allUniqueName="[Month_by_Month].[Month (Quarter)].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month].[Month (Month)]" caption="Month (Month)" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Month (Month)].[All]" allUniqueName="[Month_by_Month].[Month (Month)].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month]" caption="month" attribute="1" time="1" defaultMemberUniqueName="[Month_by_Month_CT].[month].[All]" allUniqueName="[Month_by_Month_CT].[month].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="2" memberValueDatatype="7" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_CT].[total_revenue]" caption="total_revenue" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[total_revenue].[All]" allUniqueName="[Month_by_Month_CT].[total_revenue].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="2" memberValueDatatype="5" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month (Year)]" caption="month (Year)" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[month (Year)].[All]" allUniqueName="[Month_by_Month_CT].[month (Year)].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month (Quarter)]" caption="month (Quarter)" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[month (Quarter)].[All]" allUniqueName="[Month_by_Month_CT].[month (Quarter)].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month (Month)]" caption="month (Month)" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[month (Month)].[All]" allUniqueName="[Month_by_Month_CT].[month (Month)].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month]" caption="month" attribute="1" time="1" defaultMemberUniqueName="[Month_by_Month_NY].[month].[All]" allUniqueName="[Month_by_Month_NY].[month].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="2" memberValueDatatype="7" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_NY].[total_revenue]" caption="total_revenue" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[total_revenue].[All]" allUniqueName="[Month_by_Month_NY].[total_revenue].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="2" memberValueDatatype="5" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month (Year)]" caption="month (Year)" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[month (Year)].[All]" allUniqueName="[Month_by_Month_NY].[month (Year)].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month (Quarter)]" caption="month (Quarter)" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[month (Quarter)].[All]" allUniqueName="[Month_by_Month_NY].[month (Quarter)].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month (Month)]" caption="month (Month)" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[month (Month)].[All]" allUniqueName="[Month_by_Month_NY].[month (Month)].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
-    <cacheHierarchy uniqueName="[Month_by_Month].[Month (Month Index)]" caption="Month (Month Index)" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Month (Month Index)].[All]" allUniqueName="[Month_by_Month].[Month (Month Index)].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="2" memberValueDatatype="20" unbalanced="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month (Month Index)]" caption="month (Month Index)" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[month (Month Index)].[All]" allUniqueName="[Month_by_Month_CT].[month (Month Index)].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="2" memberValueDatatype="20" unbalanced="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month (Month Index)]" caption="month (Month Index)" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[month (Month Index)].[All]" allUniqueName="[Month_by_Month_NY].[month (Month Index)].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="2" memberValueDatatype="20" unbalanced="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[__XL_Count Month_by_Month_NY]" caption="__XL_Count Month_by_Month_NY" measure="1" displayFolder="" measureGroup="Month_by_Month_NY" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[__XL_Count Month_by_Month_CT]" caption="__XL_Count Month_by_Month_CT" measure="1" displayFolder="" measureGroup="Month_by_Month_CT" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[__XL_Count Month_by_Month]" caption="__XL_Count Month_by_Month" measure="1" displayFolder="" measureGroup="Month_by_Month" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[__XL_Count Category_Percentage_CT]" caption="__XL_Count Category_Percentage_CT" measure="1" displayFolder="" measureGroup="Category_Percentage_CT" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[__XL_Count Category_Percentage_NY]" caption="__XL_Count Category_Percentage_NY" measure="1" displayFolder="" measureGroup="Category_Percentage_NY" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[__No measures defined]" caption="__No measures defined" measure="1" displayFolder="" count="0" hidden="1"/>
-    <cacheHierarchy uniqueName="[Measures].[Sum of total_revenue 2]" caption="Sum of total_revenue 2" measure="1" displayFolder="" measureGroup="Month_by_Month_NY" count="0" hidden="1">
-      <extLst>
-        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
-          <x15:cacheHierarchy aggregatedColumn="17"/>
-        </ext>
-      </extLst>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Measures].[Sum of total_revenue]" caption="Sum of total_revenue" measure="1" displayFolder="" measureGroup="Month_by_Month_CT" count="0" hidden="1">
-      <extLst>
-        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
-          <x15:cacheHierarchy aggregatedColumn="12"/>
-        </ext>
-      </extLst>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Measures].[Sum of Total_Revenue 3]" caption="Sum of Total_Revenue 3" measure="1" displayFolder="" measureGroup="Month_by_Month" count="0" hidden="1">
-      <extLst>
-        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
-          <x15:cacheHierarchy aggregatedColumn="7"/>
-        </ext>
-      </extLst>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Measures].[Sum of category_percentage]" caption="Sum of category_percentage" measure="1" displayFolder="" measureGroup="Category_Percentage_CT" count="0" hidden="1">
-      <extLst>
-        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
-          <x15:cacheHierarchy aggregatedColumn="2"/>
-        </ext>
-      </extLst>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Measures].[Sum of store_id]" caption="Sum of store_id" measure="1" displayFolder="" measureGroup="Category_Percentage_CT" count="0" hidden="1">
-      <extLst>
-        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
-          <x15:cacheHierarchy aggregatedColumn="0"/>
-        </ext>
-      </extLst>
-    </cacheHierarchy>
-    <cacheHierarchy uniqueName="[Measures].[Sum of category_percentage 2]" caption="Sum of category_percentage 2" measure="1" displayFolder="" measureGroup="Category_Percentage_NY" count="0" oneField="1" hidden="1">
-      <fieldsUsage count="1">
-        <fieldUsage x="1"/>
-      </fieldsUsage>
-      <extLst>
-        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
-          <x15:cacheHierarchy aggregatedColumn="5"/>
-        </ext>
-      </extLst>
-    </cacheHierarchy>
-  </cacheHierarchies>
-  <kpis count="0"/>
-  <dimensions count="6">
-    <dimension name="Category_Percentage_CT" uniqueName="[Category_Percentage_CT]" caption="Category_Percentage_CT"/>
-    <dimension name="Category_Percentage_NY" uniqueName="[Category_Percentage_NY]" caption="Category_Percentage_NY"/>
-    <dimension measure="1" name="Measures" uniqueName="[Measures]" caption="Measures"/>
-    <dimension name="Month_by_Month" uniqueName="[Month_by_Month]" caption="Month_by_Month"/>
-    <dimension name="Month_by_Month_CT" uniqueName="[Month_by_Month_CT]" caption="Month_by_Month_CT"/>
-    <dimension name="Month_by_Month_NY" uniqueName="[Month_by_Month_NY]" caption="Month_by_Month_NY"/>
-  </dimensions>
-  <measureGroups count="5">
-    <measureGroup name="Category_Percentage_CT" caption="Category_Percentage_CT"/>
-    <measureGroup name="Category_Percentage_NY" caption="Category_Percentage_NY"/>
-    <measureGroup name="Month_by_Month" caption="Month_by_Month"/>
-    <measureGroup name="Month_by_Month_CT" caption="Month_by_Month_CT"/>
-    <measureGroup name="Month_by_Month_NY" caption="Month_by_Month_NY"/>
-  </measureGroups>
-  <maps count="5">
-    <map measureGroup="0" dimension="0"/>
-    <map measureGroup="1" dimension="1"/>
-    <map measureGroup="2" dimension="3"/>
-    <map measureGroup="3" dimension="4"/>
-    <map measureGroup="4" dimension="5"/>
-  </maps>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition supportSubqueryNonVisual="1" supportSubqueryCalcMem="1" supportAddCalcMems="1"/>
-    </ext>
-  </extLst>
-</pivotCacheDefinition>
-</file>
-
-<file path=xl/pivotCache/pivotCacheDefinition5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="Chantal Lee" refreshedDate="46143.027661689812" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{9E281A56-8DD1-4B0E-A308-F91AD1A8ADED}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="Chantal Lee" refreshedDate="46143.111483333334" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{9E281A56-8DD1-4B0E-A308-F91AD1A8ADED}">
   <cacheSource type="external" connectionId="6"/>
   <cacheFields count="5">
     <cacheField name="[Measures].[Sum of Total_Revenue 3]" caption="Sum of Total_Revenue 3" numFmtId="0" hierarchy="32" level="32767"/>
@@ -16781,6 +17516,653 @@
       </extLst>
     </cacheHierarchy>
     <cacheHierarchy uniqueName="[Measures].[Sum of category_percentage 2]" caption="Sum of category_percentage 2" measure="1" displayFolder="" measureGroup="Category_Percentage_NY" count="0" hidden="1">
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="5"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+  </cacheHierarchies>
+  <kpis count="0"/>
+  <dimensions count="6">
+    <dimension name="Category_Percentage_CT" uniqueName="[Category_Percentage_CT]" caption="Category_Percentage_CT"/>
+    <dimension name="Category_Percentage_NY" uniqueName="[Category_Percentage_NY]" caption="Category_Percentage_NY"/>
+    <dimension measure="1" name="Measures" uniqueName="[Measures]" caption="Measures"/>
+    <dimension name="Month_by_Month" uniqueName="[Month_by_Month]" caption="Month_by_Month"/>
+    <dimension name="Month_by_Month_CT" uniqueName="[Month_by_Month_CT]" caption="Month_by_Month_CT"/>
+    <dimension name="Month_by_Month_NY" uniqueName="[Month_by_Month_NY]" caption="Month_by_Month_NY"/>
+  </dimensions>
+  <measureGroups count="5">
+    <measureGroup name="Category_Percentage_CT" caption="Category_Percentage_CT"/>
+    <measureGroup name="Category_Percentage_NY" caption="Category_Percentage_NY"/>
+    <measureGroup name="Month_by_Month" caption="Month_by_Month"/>
+    <measureGroup name="Month_by_Month_CT" caption="Month_by_Month_CT"/>
+    <measureGroup name="Month_by_Month_NY" caption="Month_by_Month_NY"/>
+  </measureGroups>
+  <maps count="5">
+    <map measureGroup="0" dimension="0"/>
+    <map measureGroup="1" dimension="1"/>
+    <map measureGroup="2" dimension="3"/>
+    <map measureGroup="3" dimension="4"/>
+    <map measureGroup="4" dimension="5"/>
+  </maps>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition supportSubqueryNonVisual="1" supportSubqueryCalcMem="1" supportAddCalcMems="1"/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="Chantal Lee" refreshedDate="46143.12008252315" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{B0A6EEAC-EAE3-4C7C-BC5A-70188D13667D}">
+  <cacheSource type="external" connectionId="6"/>
+  <cacheFields count="5">
+    <cacheField name="[Month_by_Month_CT].[month].[month]" caption="month" numFmtId="0" hierarchy="11" level="1">
+      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2024-09-01T00:00:00" maxDate="2024-09-02T00:00:00" count="1">
+        <d v="2024-09-01T00:00:00"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="[Month_by_Month_CT].[month (Month)].[month (Month)]" caption="month (Month)" numFmtId="0" hierarchy="15" level="1">
+      <sharedItems count="1">
+        <s v="Sep"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="[Month_by_Month_CT].[month (Quarter)].[month (Quarter)]" caption="month (Quarter)" numFmtId="0" hierarchy="14" level="1">
+      <sharedItems count="1">
+        <s v="Qtr3"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="[Month_by_Month_CT].[month (Year)].[month (Year)]" caption="month (Year)" numFmtId="0" hierarchy="13" level="1">
+      <sharedItems count="4">
+        <s v="2022"/>
+        <s v="2023"/>
+        <s v="2024"/>
+        <s v="2025"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="[Measures].[Sum of total_revenue]" caption="Sum of total_revenue" numFmtId="0" hierarchy="31" level="32767"/>
+  </cacheFields>
+  <cacheHierarchies count="36">
+    <cacheHierarchy uniqueName="[Category_Percentage_CT].[store_id]" caption="store_id" attribute="1" defaultMemberUniqueName="[Category_Percentage_CT].[store_id].[All]" allUniqueName="[Category_Percentage_CT].[store_id].[All]" dimensionUniqueName="[Category_Percentage_CT]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Category_Percentage_CT].[category]" caption="category" attribute="1" defaultMemberUniqueName="[Category_Percentage_CT].[category].[All]" allUniqueName="[Category_Percentage_CT].[category].[All]" dimensionUniqueName="[Category_Percentage_CT]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Category_Percentage_CT].[category_percentage]" caption="category_percentage" attribute="1" defaultMemberUniqueName="[Category_Percentage_CT].[category_percentage].[All]" allUniqueName="[Category_Percentage_CT].[category_percentage].[All]" dimensionUniqueName="[Category_Percentage_CT]" displayFolder="" count="0" memberValueDatatype="5" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Category_Percentage_NY].[store_id]" caption="store_id" attribute="1" defaultMemberUniqueName="[Category_Percentage_NY].[store_id].[All]" allUniqueName="[Category_Percentage_NY].[store_id].[All]" dimensionUniqueName="[Category_Percentage_NY]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Category_Percentage_NY].[category]" caption="category" attribute="1" defaultMemberUniqueName="[Category_Percentage_NY].[category].[All]" allUniqueName="[Category_Percentage_NY].[category].[All]" dimensionUniqueName="[Category_Percentage_NY]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Category_Percentage_NY].[category_percentage]" caption="category_percentage" attribute="1" defaultMemberUniqueName="[Category_Percentage_NY].[category_percentage].[All]" allUniqueName="[Category_Percentage_NY].[category_percentage].[All]" dimensionUniqueName="[Category_Percentage_NY]" displayFolder="" count="0" memberValueDatatype="5" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month].[Month]" caption="Month" attribute="1" time="1" defaultMemberUniqueName="[Month_by_Month].[Month].[All]" allUniqueName="[Month_by_Month].[Month].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="0" memberValueDatatype="7" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month].[Total_Revenue]" caption="Total_Revenue" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Total_Revenue].[All]" allUniqueName="[Month_by_Month].[Total_Revenue].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="0" memberValueDatatype="5" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month].[Month (Year)]" caption="Month (Year)" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Month (Year)].[All]" allUniqueName="[Month_by_Month].[Month (Year)].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month].[Month (Quarter)]" caption="Month (Quarter)" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Month (Quarter)].[All]" allUniqueName="[Month_by_Month].[Month (Quarter)].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month].[Month (Month)]" caption="Month (Month)" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Month (Month)].[All]" allUniqueName="[Month_by_Month].[Month (Month)].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month]" caption="month" attribute="1" time="1" defaultMemberUniqueName="[Month_by_Month_CT].[month].[All]" allUniqueName="[Month_by_Month_CT].[month].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="2" memberValueDatatype="7" unbalanced="0">
+      <fieldsUsage count="2">
+        <fieldUsage x="-1"/>
+        <fieldUsage x="0"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Month_by_Month_CT].[total_revenue]" caption="total_revenue" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[total_revenue].[All]" allUniqueName="[Month_by_Month_CT].[total_revenue].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="0" memberValueDatatype="5" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month (Year)]" caption="month (Year)" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[month (Year)].[All]" allUniqueName="[Month_by_Month_CT].[month (Year)].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0">
+      <fieldsUsage count="2">
+        <fieldUsage x="-1"/>
+        <fieldUsage x="3"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month (Quarter)]" caption="month (Quarter)" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[month (Quarter)].[All]" allUniqueName="[Month_by_Month_CT].[month (Quarter)].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0">
+      <fieldsUsage count="2">
+        <fieldUsage x="-1"/>
+        <fieldUsage x="2"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month (Month)]" caption="month (Month)" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[month (Month)].[All]" allUniqueName="[Month_by_Month_CT].[month (Month)].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0">
+      <fieldsUsage count="2">
+        <fieldUsage x="-1"/>
+        <fieldUsage x="1"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month]" caption="month" attribute="1" time="1" defaultMemberUniqueName="[Month_by_Month_NY].[month].[All]" allUniqueName="[Month_by_Month_NY].[month].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="0" memberValueDatatype="7" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_NY].[total_revenue]" caption="total_revenue" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[total_revenue].[All]" allUniqueName="[Month_by_Month_NY].[total_revenue].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="0" memberValueDatatype="5" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month (Year)]" caption="month (Year)" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[month (Year)].[All]" allUniqueName="[Month_by_Month_NY].[month (Year)].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month (Quarter)]" caption="month (Quarter)" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[month (Quarter)].[All]" allUniqueName="[Month_by_Month_NY].[month (Quarter)].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month (Month)]" caption="month (Month)" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[month (Month)].[All]" allUniqueName="[Month_by_Month_NY].[month (Month)].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month].[Month (Month Index)]" caption="Month (Month Index)" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Month (Month Index)].[All]" allUniqueName="[Month_by_Month].[Month (Month Index)].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month (Month Index)]" caption="month (Month Index)" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[month (Month Index)].[All]" allUniqueName="[Month_by_Month_CT].[month (Month Index)].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month (Month Index)]" caption="month (Month Index)" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[month (Month Index)].[All]" allUniqueName="[Month_by_Month_NY].[month (Month Index)].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__XL_Count Month_by_Month_NY]" caption="__XL_Count Month_by_Month_NY" measure="1" displayFolder="" measureGroup="Month_by_Month_NY" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__XL_Count Month_by_Month_CT]" caption="__XL_Count Month_by_Month_CT" measure="1" displayFolder="" measureGroup="Month_by_Month_CT" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__XL_Count Month_by_Month]" caption="__XL_Count Month_by_Month" measure="1" displayFolder="" measureGroup="Month_by_Month" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__XL_Count Category_Percentage_CT]" caption="__XL_Count Category_Percentage_CT" measure="1" displayFolder="" measureGroup="Category_Percentage_CT" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__XL_Count Category_Percentage_NY]" caption="__XL_Count Category_Percentage_NY" measure="1" displayFolder="" measureGroup="Category_Percentage_NY" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__No measures defined]" caption="__No measures defined" measure="1" displayFolder="" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[Sum of total_revenue 2]" caption="Sum of total_revenue 2" measure="1" displayFolder="" measureGroup="Month_by_Month_NY" count="0" hidden="1">
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="17"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[Sum of total_revenue]" caption="Sum of total_revenue" measure="1" displayFolder="" measureGroup="Month_by_Month_CT" count="0" oneField="1" hidden="1">
+      <fieldsUsage count="1">
+        <fieldUsage x="4"/>
+      </fieldsUsage>
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="12"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[Sum of Total_Revenue 3]" caption="Sum of Total_Revenue 3" measure="1" displayFolder="" measureGroup="Month_by_Month" count="0" hidden="1">
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="7"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[Sum of category_percentage]" caption="Sum of category_percentage" measure="1" displayFolder="" measureGroup="Category_Percentage_CT" count="0" hidden="1">
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="2"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[Sum of store_id]" caption="Sum of store_id" measure="1" displayFolder="" measureGroup="Category_Percentage_CT" count="0" hidden="1">
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="0"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[Sum of category_percentage 2]" caption="Sum of category_percentage 2" measure="1" displayFolder="" measureGroup="Category_Percentage_NY" count="0" hidden="1">
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="5"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+  </cacheHierarchies>
+  <kpis count="0"/>
+  <dimensions count="6">
+    <dimension name="Category_Percentage_CT" uniqueName="[Category_Percentage_CT]" caption="Category_Percentage_CT"/>
+    <dimension name="Category_Percentage_NY" uniqueName="[Category_Percentage_NY]" caption="Category_Percentage_NY"/>
+    <dimension measure="1" name="Measures" uniqueName="[Measures]" caption="Measures"/>
+    <dimension name="Month_by_Month" uniqueName="[Month_by_Month]" caption="Month_by_Month"/>
+    <dimension name="Month_by_Month_CT" uniqueName="[Month_by_Month_CT]" caption="Month_by_Month_CT"/>
+    <dimension name="Month_by_Month_NY" uniqueName="[Month_by_Month_NY]" caption="Month_by_Month_NY"/>
+  </dimensions>
+  <measureGroups count="5">
+    <measureGroup name="Category_Percentage_CT" caption="Category_Percentage_CT"/>
+    <measureGroup name="Category_Percentage_NY" caption="Category_Percentage_NY"/>
+    <measureGroup name="Month_by_Month" caption="Month_by_Month"/>
+    <measureGroup name="Month_by_Month_CT" caption="Month_by_Month_CT"/>
+    <measureGroup name="Month_by_Month_NY" caption="Month_by_Month_NY"/>
+  </measureGroups>
+  <maps count="5">
+    <map measureGroup="0" dimension="0"/>
+    <map measureGroup="1" dimension="1"/>
+    <map measureGroup="2" dimension="3"/>
+    <map measureGroup="3" dimension="4"/>
+    <map measureGroup="4" dimension="5"/>
+  </maps>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition supportSubqueryNonVisual="1" supportSubqueryCalcMem="1" supportAddCalcMems="1"/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="Chantal Lee" refreshedDate="46143.120145833331" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{3728C892-97BF-4BD3-8C3A-33A379001046}">
+  <cacheSource type="external" connectionId="6"/>
+  <cacheFields count="5">
+    <cacheField name="[Month_by_Month_NY].[month].[month]" caption="month" numFmtId="0" hierarchy="16" level="1">
+      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2022-01-01T00:00:00" maxDate="2022-01-02T00:00:00" count="1">
+        <d v="2022-01-01T00:00:00"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="[Month_by_Month_NY].[month (Month)].[month (Month)]" caption="month (Month)" numFmtId="0" hierarchy="20" level="1">
+      <sharedItems count="3">
+        <s v="Jan"/>
+        <s v="Feb"/>
+        <s v="Mar"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="[Month_by_Month_NY].[month (Quarter)].[month (Quarter)]" caption="month (Quarter)" numFmtId="0" hierarchy="19" level="1">
+      <sharedItems count="4">
+        <s v="Qtr1"/>
+        <s v="Qtr2"/>
+        <s v="Qtr3"/>
+        <s v="Qtr4"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="[Month_by_Month_NY].[month (Year)].[month (Year)]" caption="month (Year)" numFmtId="0" hierarchy="18" level="1">
+      <sharedItems count="4">
+        <s v="2022"/>
+        <s v="2023"/>
+        <s v="2024"/>
+        <s v="2025"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="[Measures].[Sum of total_revenue 2]" caption="Sum of total_revenue 2" numFmtId="0" hierarchy="30" level="32767"/>
+  </cacheFields>
+  <cacheHierarchies count="36">
+    <cacheHierarchy uniqueName="[Category_Percentage_CT].[store_id]" caption="store_id" attribute="1" defaultMemberUniqueName="[Category_Percentage_CT].[store_id].[All]" allUniqueName="[Category_Percentage_CT].[store_id].[All]" dimensionUniqueName="[Category_Percentage_CT]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Category_Percentage_CT].[category]" caption="category" attribute="1" defaultMemberUniqueName="[Category_Percentage_CT].[category].[All]" allUniqueName="[Category_Percentage_CT].[category].[All]" dimensionUniqueName="[Category_Percentage_CT]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Category_Percentage_CT].[category_percentage]" caption="category_percentage" attribute="1" defaultMemberUniqueName="[Category_Percentage_CT].[category_percentage].[All]" allUniqueName="[Category_Percentage_CT].[category_percentage].[All]" dimensionUniqueName="[Category_Percentage_CT]" displayFolder="" count="0" memberValueDatatype="5" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Category_Percentage_NY].[store_id]" caption="store_id" attribute="1" defaultMemberUniqueName="[Category_Percentage_NY].[store_id].[All]" allUniqueName="[Category_Percentage_NY].[store_id].[All]" dimensionUniqueName="[Category_Percentage_NY]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Category_Percentage_NY].[category]" caption="category" attribute="1" defaultMemberUniqueName="[Category_Percentage_NY].[category].[All]" allUniqueName="[Category_Percentage_NY].[category].[All]" dimensionUniqueName="[Category_Percentage_NY]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Category_Percentage_NY].[category_percentage]" caption="category_percentage" attribute="1" defaultMemberUniqueName="[Category_Percentage_NY].[category_percentage].[All]" allUniqueName="[Category_Percentage_NY].[category_percentage].[All]" dimensionUniqueName="[Category_Percentage_NY]" displayFolder="" count="0" memberValueDatatype="5" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month].[Month]" caption="Month" attribute="1" time="1" defaultMemberUniqueName="[Month_by_Month].[Month].[All]" allUniqueName="[Month_by_Month].[Month].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="0" memberValueDatatype="7" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month].[Total_Revenue]" caption="Total_Revenue" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Total_Revenue].[All]" allUniqueName="[Month_by_Month].[Total_Revenue].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="0" memberValueDatatype="5" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month].[Month (Year)]" caption="Month (Year)" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Month (Year)].[All]" allUniqueName="[Month_by_Month].[Month (Year)].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month].[Month (Quarter)]" caption="Month (Quarter)" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Month (Quarter)].[All]" allUniqueName="[Month_by_Month].[Month (Quarter)].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month].[Month (Month)]" caption="Month (Month)" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Month (Month)].[All]" allUniqueName="[Month_by_Month].[Month (Month)].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month]" caption="month" attribute="1" time="1" defaultMemberUniqueName="[Month_by_Month_CT].[month].[All]" allUniqueName="[Month_by_Month_CT].[month].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="0" memberValueDatatype="7" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_CT].[total_revenue]" caption="total_revenue" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[total_revenue].[All]" allUniqueName="[Month_by_Month_CT].[total_revenue].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="0" memberValueDatatype="5" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month (Year)]" caption="month (Year)" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[month (Year)].[All]" allUniqueName="[Month_by_Month_CT].[month (Year)].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month (Quarter)]" caption="month (Quarter)" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[month (Quarter)].[All]" allUniqueName="[Month_by_Month_CT].[month (Quarter)].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month (Month)]" caption="month (Month)" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[month (Month)].[All]" allUniqueName="[Month_by_Month_CT].[month (Month)].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="0" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month]" caption="month" attribute="1" time="1" defaultMemberUniqueName="[Month_by_Month_NY].[month].[All]" allUniqueName="[Month_by_Month_NY].[month].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="2" memberValueDatatype="7" unbalanced="0">
+      <fieldsUsage count="2">
+        <fieldUsage x="-1"/>
+        <fieldUsage x="0"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Month_by_Month_NY].[total_revenue]" caption="total_revenue" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[total_revenue].[All]" allUniqueName="[Month_by_Month_NY].[total_revenue].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="0" memberValueDatatype="5" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month (Year)]" caption="month (Year)" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[month (Year)].[All]" allUniqueName="[Month_by_Month_NY].[month (Year)].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0">
+      <fieldsUsage count="2">
+        <fieldUsage x="-1"/>
+        <fieldUsage x="3"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month (Quarter)]" caption="month (Quarter)" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[month (Quarter)].[All]" allUniqueName="[Month_by_Month_NY].[month (Quarter)].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0">
+      <fieldsUsage count="2">
+        <fieldUsage x="-1"/>
+        <fieldUsage x="2"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month (Month)]" caption="month (Month)" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[month (Month)].[All]" allUniqueName="[Month_by_Month_NY].[month (Month)].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0">
+      <fieldsUsage count="2">
+        <fieldUsage x="-1"/>
+        <fieldUsage x="1"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Month_by_Month].[Month (Month Index)]" caption="Month (Month Index)" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Month (Month Index)].[All]" allUniqueName="[Month_by_Month].[Month (Month Index)].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month (Month Index)]" caption="month (Month Index)" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[month (Month Index)].[All]" allUniqueName="[Month_by_Month_CT].[month (Month Index)].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month (Month Index)]" caption="month (Month Index)" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[month (Month Index)].[All]" allUniqueName="[Month_by_Month_NY].[month (Month Index)].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="0" memberValueDatatype="20" unbalanced="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__XL_Count Month_by_Month_NY]" caption="__XL_Count Month_by_Month_NY" measure="1" displayFolder="" measureGroup="Month_by_Month_NY" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__XL_Count Month_by_Month_CT]" caption="__XL_Count Month_by_Month_CT" measure="1" displayFolder="" measureGroup="Month_by_Month_CT" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__XL_Count Month_by_Month]" caption="__XL_Count Month_by_Month" measure="1" displayFolder="" measureGroup="Month_by_Month" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__XL_Count Category_Percentage_CT]" caption="__XL_Count Category_Percentage_CT" measure="1" displayFolder="" measureGroup="Category_Percentage_CT" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__XL_Count Category_Percentage_NY]" caption="__XL_Count Category_Percentage_NY" measure="1" displayFolder="" measureGroup="Category_Percentage_NY" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__No measures defined]" caption="__No measures defined" measure="1" displayFolder="" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[Sum of total_revenue 2]" caption="Sum of total_revenue 2" measure="1" displayFolder="" measureGroup="Month_by_Month_NY" count="0" oneField="1" hidden="1">
+      <fieldsUsage count="1">
+        <fieldUsage x="4"/>
+      </fieldsUsage>
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="17"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[Sum of total_revenue]" caption="Sum of total_revenue" measure="1" displayFolder="" measureGroup="Month_by_Month_CT" count="0" hidden="1">
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="12"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[Sum of Total_Revenue 3]" caption="Sum of Total_Revenue 3" measure="1" displayFolder="" measureGroup="Month_by_Month" count="0" hidden="1">
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="7"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[Sum of category_percentage]" caption="Sum of category_percentage" measure="1" displayFolder="" measureGroup="Category_Percentage_CT" count="0" hidden="1">
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="2"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[Sum of store_id]" caption="Sum of store_id" measure="1" displayFolder="" measureGroup="Category_Percentage_CT" count="0" hidden="1">
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="0"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[Sum of category_percentage 2]" caption="Sum of category_percentage 2" measure="1" displayFolder="" measureGroup="Category_Percentage_NY" count="0" hidden="1">
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="5"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+  </cacheHierarchies>
+  <kpis count="0"/>
+  <dimensions count="6">
+    <dimension name="Category_Percentage_CT" uniqueName="[Category_Percentage_CT]" caption="Category_Percentage_CT"/>
+    <dimension name="Category_Percentage_NY" uniqueName="[Category_Percentage_NY]" caption="Category_Percentage_NY"/>
+    <dimension measure="1" name="Measures" uniqueName="[Measures]" caption="Measures"/>
+    <dimension name="Month_by_Month" uniqueName="[Month_by_Month]" caption="Month_by_Month"/>
+    <dimension name="Month_by_Month_CT" uniqueName="[Month_by_Month_CT]" caption="Month_by_Month_CT"/>
+    <dimension name="Month_by_Month_NY" uniqueName="[Month_by_Month_NY]" caption="Month_by_Month_NY"/>
+  </dimensions>
+  <measureGroups count="5">
+    <measureGroup name="Category_Percentage_CT" caption="Category_Percentage_CT"/>
+    <measureGroup name="Category_Percentage_NY" caption="Category_Percentage_NY"/>
+    <measureGroup name="Month_by_Month" caption="Month_by_Month"/>
+    <measureGroup name="Month_by_Month_CT" caption="Month_by_Month_CT"/>
+    <measureGroup name="Month_by_Month_NY" caption="Month_by_Month_NY"/>
+  </measureGroups>
+  <maps count="5">
+    <map measureGroup="0" dimension="0"/>
+    <map measureGroup="1" dimension="1"/>
+    <map measureGroup="2" dimension="3"/>
+    <map measureGroup="3" dimension="4"/>
+    <map measureGroup="4" dimension="5"/>
+  </maps>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition supportSubqueryNonVisual="1" supportSubqueryCalcMem="1" supportAddCalcMems="1"/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="Chantal Lee" refreshedDate="46143.120541898148" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{9CCA98CC-7441-4E2D-BA36-575067284E5B}">
+  <cacheSource type="external" connectionId="6"/>
+  <cacheFields count="3">
+    <cacheField name="[Category_Percentage_CT].[category].[category]" caption="category" numFmtId="0" hierarchy="1" level="1">
+      <sharedItems count="6">
+        <s v="Apparel and Merchandise"/>
+        <s v="Art Supplies"/>
+        <s v="Books (General)"/>
+        <s v="Stationery and Supplies"/>
+        <s v="Technology &amp; Accessories"/>
+        <s v="Textbooks"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="[Measures].[Sum of category_percentage]" caption="Sum of category_percentage" numFmtId="0" hierarchy="33" level="32767"/>
+    <cacheField name="[Category_Percentage_CT].[store_id].[store_id]" caption="store_id" numFmtId="0" level="1">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="865" maxValue="872" count="8">
+        <n v="870"/>
+        <n v="871" u="1"/>
+        <n v="865" u="1"/>
+        <n v="866" u="1"/>
+        <n v="868" u="1"/>
+        <n v="867" u="1"/>
+        <n v="869" u="1"/>
+        <n v="872" u="1"/>
+      </sharedItems>
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{4F2E5C28-24EA-4eb8-9CBF-B6C8F9C3D259}">
+          <x15:cachedUniqueNames>
+            <x15:cachedUniqueName index="0" name="[Category_Percentage_CT].[store_id].&amp;[870]"/>
+            <x15:cachedUniqueName index="1" name="[Category_Percentage_CT].[store_id].&amp;[871]"/>
+            <x15:cachedUniqueName index="2" name="[Category_Percentage_CT].[store_id].&amp;[865]"/>
+            <x15:cachedUniqueName index="3" name="[Category_Percentage_CT].[store_id].&amp;[866]"/>
+            <x15:cachedUniqueName index="4" name="[Category_Percentage_CT].[store_id].&amp;[868]"/>
+            <x15:cachedUniqueName index="5" name="[Category_Percentage_CT].[store_id].&amp;[867]"/>
+            <x15:cachedUniqueName index="6" name="[Category_Percentage_CT].[store_id].&amp;[869]"/>
+            <x15:cachedUniqueName index="7" name="[Category_Percentage_CT].[store_id].&amp;[872]"/>
+          </x15:cachedUniqueNames>
+        </ext>
+      </extLst>
+    </cacheField>
+  </cacheFields>
+  <cacheHierarchies count="36">
+    <cacheHierarchy uniqueName="[Category_Percentage_CT].[store_id]" caption="store_id" attribute="1" defaultMemberUniqueName="[Category_Percentage_CT].[store_id].[All]" allUniqueName="[Category_Percentage_CT].[store_id].[All]" dimensionUniqueName="[Category_Percentage_CT]" displayFolder="" count="2" memberValueDatatype="20" unbalanced="0">
+      <fieldsUsage count="2">
+        <fieldUsage x="-1"/>
+        <fieldUsage x="2"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Category_Percentage_CT].[category]" caption="category" attribute="1" defaultMemberUniqueName="[Category_Percentage_CT].[category].[All]" allUniqueName="[Category_Percentage_CT].[category].[All]" dimensionUniqueName="[Category_Percentage_CT]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0">
+      <fieldsUsage count="2">
+        <fieldUsage x="-1"/>
+        <fieldUsage x="0"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Category_Percentage_CT].[category_percentage]" caption="category_percentage" attribute="1" defaultMemberUniqueName="[Category_Percentage_CT].[category_percentage].[All]" allUniqueName="[Category_Percentage_CT].[category_percentage].[All]" dimensionUniqueName="[Category_Percentage_CT]" displayFolder="" count="2" memberValueDatatype="5" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Category_Percentage_NY].[store_id]" caption="store_id" attribute="1" defaultMemberUniqueName="[Category_Percentage_NY].[store_id].[All]" allUniqueName="[Category_Percentage_NY].[store_id].[All]" dimensionUniqueName="[Category_Percentage_NY]" displayFolder="" count="2" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Category_Percentage_NY].[category]" caption="category" attribute="1" defaultMemberUniqueName="[Category_Percentage_NY].[category].[All]" allUniqueName="[Category_Percentage_NY].[category].[All]" dimensionUniqueName="[Category_Percentage_NY]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Category_Percentage_NY].[category_percentage]" caption="category_percentage" attribute="1" defaultMemberUniqueName="[Category_Percentage_NY].[category_percentage].[All]" allUniqueName="[Category_Percentage_NY].[category_percentage].[All]" dimensionUniqueName="[Category_Percentage_NY]" displayFolder="" count="2" memberValueDatatype="5" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month].[Month]" caption="Month" attribute="1" time="1" defaultMemberUniqueName="[Month_by_Month].[Month].[All]" allUniqueName="[Month_by_Month].[Month].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="2" memberValueDatatype="7" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month].[Total_Revenue]" caption="Total_Revenue" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Total_Revenue].[All]" allUniqueName="[Month_by_Month].[Total_Revenue].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="2" memberValueDatatype="5" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month].[Month (Year)]" caption="Month (Year)" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Month (Year)].[All]" allUniqueName="[Month_by_Month].[Month (Year)].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month].[Month (Quarter)]" caption="Month (Quarter)" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Month (Quarter)].[All]" allUniqueName="[Month_by_Month].[Month (Quarter)].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month].[Month (Month)]" caption="Month (Month)" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Month (Month)].[All]" allUniqueName="[Month_by_Month].[Month (Month)].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month]" caption="month" attribute="1" time="1" defaultMemberUniqueName="[Month_by_Month_CT].[month].[All]" allUniqueName="[Month_by_Month_CT].[month].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="2" memberValueDatatype="7" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_CT].[total_revenue]" caption="total_revenue" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[total_revenue].[All]" allUniqueName="[Month_by_Month_CT].[total_revenue].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="2" memberValueDatatype="5" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month (Year)]" caption="month (Year)" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[month (Year)].[All]" allUniqueName="[Month_by_Month_CT].[month (Year)].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month (Quarter)]" caption="month (Quarter)" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[month (Quarter)].[All]" allUniqueName="[Month_by_Month_CT].[month (Quarter)].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month (Month)]" caption="month (Month)" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[month (Month)].[All]" allUniqueName="[Month_by_Month_CT].[month (Month)].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month]" caption="month" attribute="1" time="1" defaultMemberUniqueName="[Month_by_Month_NY].[month].[All]" allUniqueName="[Month_by_Month_NY].[month].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="2" memberValueDatatype="7" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_NY].[total_revenue]" caption="total_revenue" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[total_revenue].[All]" allUniqueName="[Month_by_Month_NY].[total_revenue].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="2" memberValueDatatype="5" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month (Year)]" caption="month (Year)" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[month (Year)].[All]" allUniqueName="[Month_by_Month_NY].[month (Year)].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month (Quarter)]" caption="month (Quarter)" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[month (Quarter)].[All]" allUniqueName="[Month_by_Month_NY].[month (Quarter)].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month (Month)]" caption="month (Month)" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[month (Month)].[All]" allUniqueName="[Month_by_Month_NY].[month (Month)].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month].[Month (Month Index)]" caption="Month (Month Index)" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Month (Month Index)].[All]" allUniqueName="[Month_by_Month].[Month (Month Index)].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="2" memberValueDatatype="20" unbalanced="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month (Month Index)]" caption="month (Month Index)" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[month (Month Index)].[All]" allUniqueName="[Month_by_Month_CT].[month (Month Index)].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="2" memberValueDatatype="20" unbalanced="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month (Month Index)]" caption="month (Month Index)" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[month (Month Index)].[All]" allUniqueName="[Month_by_Month_NY].[month (Month Index)].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="2" memberValueDatatype="20" unbalanced="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__XL_Count Month_by_Month_NY]" caption="__XL_Count Month_by_Month_NY" measure="1" displayFolder="" measureGroup="Month_by_Month_NY" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__XL_Count Month_by_Month_CT]" caption="__XL_Count Month_by_Month_CT" measure="1" displayFolder="" measureGroup="Month_by_Month_CT" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__XL_Count Month_by_Month]" caption="__XL_Count Month_by_Month" measure="1" displayFolder="" measureGroup="Month_by_Month" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__XL_Count Category_Percentage_CT]" caption="__XL_Count Category_Percentage_CT" measure="1" displayFolder="" measureGroup="Category_Percentage_CT" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__XL_Count Category_Percentage_NY]" caption="__XL_Count Category_Percentage_NY" measure="1" displayFolder="" measureGroup="Category_Percentage_NY" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__No measures defined]" caption="__No measures defined" measure="1" displayFolder="" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[Sum of total_revenue 2]" caption="Sum of total_revenue 2" measure="1" displayFolder="" measureGroup="Month_by_Month_NY" count="0" hidden="1">
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="17"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[Sum of total_revenue]" caption="Sum of total_revenue" measure="1" displayFolder="" measureGroup="Month_by_Month_CT" count="0" hidden="1">
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="12"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[Sum of Total_Revenue 3]" caption="Sum of Total_Revenue 3" measure="1" displayFolder="" measureGroup="Month_by_Month" count="0" hidden="1">
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="7"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[Sum of category_percentage]" caption="Sum of category_percentage" measure="1" displayFolder="" measureGroup="Category_Percentage_CT" count="0" oneField="1" hidden="1">
+      <fieldsUsage count="1">
+        <fieldUsage x="1"/>
+      </fieldsUsage>
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="2"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[Sum of store_id]" caption="Sum of store_id" measure="1" displayFolder="" measureGroup="Category_Percentage_CT" count="0" hidden="1">
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="0"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[Sum of category_percentage 2]" caption="Sum of category_percentage 2" measure="1" displayFolder="" measureGroup="Category_Percentage_NY" count="0" hidden="1">
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="5"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+  </cacheHierarchies>
+  <kpis count="0"/>
+  <dimensions count="6">
+    <dimension name="Category_Percentage_CT" uniqueName="[Category_Percentage_CT]" caption="Category_Percentage_CT"/>
+    <dimension name="Category_Percentage_NY" uniqueName="[Category_Percentage_NY]" caption="Category_Percentage_NY"/>
+    <dimension measure="1" name="Measures" uniqueName="[Measures]" caption="Measures"/>
+    <dimension name="Month_by_Month" uniqueName="[Month_by_Month]" caption="Month_by_Month"/>
+    <dimension name="Month_by_Month_CT" uniqueName="[Month_by_Month_CT]" caption="Month_by_Month_CT"/>
+    <dimension name="Month_by_Month_NY" uniqueName="[Month_by_Month_NY]" caption="Month_by_Month_NY"/>
+  </dimensions>
+  <measureGroups count="5">
+    <measureGroup name="Category_Percentage_CT" caption="Category_Percentage_CT"/>
+    <measureGroup name="Category_Percentage_NY" caption="Category_Percentage_NY"/>
+    <measureGroup name="Month_by_Month" caption="Month_by_Month"/>
+    <measureGroup name="Month_by_Month_CT" caption="Month_by_Month_CT"/>
+    <measureGroup name="Month_by_Month_NY" caption="Month_by_Month_NY"/>
+  </measureGroups>
+  <maps count="5">
+    <map measureGroup="0" dimension="0"/>
+    <map measureGroup="1" dimension="1"/>
+    <map measureGroup="2" dimension="3"/>
+    <map measureGroup="3" dimension="4"/>
+    <map measureGroup="4" dimension="5"/>
+  </maps>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition supportSubqueryNonVisual="1" supportSubqueryCalcMem="1" supportAddCalcMems="1"/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="Chantal Lee" refreshedDate="46143.120781597223" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{0CC7DB6F-F048-4B9F-B9D9-C2E5CD0C5F47}">
+  <cacheSource type="external" connectionId="6"/>
+  <cacheFields count="3">
+    <cacheField name="[Category_Percentage_NY].[store_id].[store_id]" caption="store_id" numFmtId="0" hierarchy="3" level="1">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="840" maxValue="851" count="12">
+        <n v="850"/>
+        <n v="851" u="1"/>
+        <n v="846" u="1"/>
+        <n v="847" u="1"/>
+        <n v="840" u="1"/>
+        <n v="841" u="1"/>
+        <n v="842" u="1"/>
+        <n v="843" u="1"/>
+        <n v="844" u="1"/>
+        <n v="845" u="1"/>
+        <n v="848" u="1"/>
+        <n v="849" u="1"/>
+      </sharedItems>
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{4F2E5C28-24EA-4eb8-9CBF-B6C8F9C3D259}">
+          <x15:cachedUniqueNames>
+            <x15:cachedUniqueName index="0" name="[Category_Percentage_NY].[store_id].&amp;[850]"/>
+            <x15:cachedUniqueName index="1" name="[Category_Percentage_NY].[store_id].&amp;[851]"/>
+            <x15:cachedUniqueName index="2" name="[Category_Percentage_NY].[store_id].&amp;[846]"/>
+            <x15:cachedUniqueName index="3" name="[Category_Percentage_NY].[store_id].&amp;[847]"/>
+            <x15:cachedUniqueName index="4" name="[Category_Percentage_NY].[store_id].&amp;[840]"/>
+            <x15:cachedUniqueName index="5" name="[Category_Percentage_NY].[store_id].&amp;[841]"/>
+            <x15:cachedUniqueName index="6" name="[Category_Percentage_NY].[store_id].&amp;[842]"/>
+            <x15:cachedUniqueName index="7" name="[Category_Percentage_NY].[store_id].&amp;[843]"/>
+            <x15:cachedUniqueName index="8" name="[Category_Percentage_NY].[store_id].&amp;[844]"/>
+            <x15:cachedUniqueName index="9" name="[Category_Percentage_NY].[store_id].&amp;[845]"/>
+            <x15:cachedUniqueName index="10" name="[Category_Percentage_NY].[store_id].&amp;[848]"/>
+            <x15:cachedUniqueName index="11" name="[Category_Percentage_NY].[store_id].&amp;[849]"/>
+          </x15:cachedUniqueNames>
+        </ext>
+      </extLst>
+    </cacheField>
+    <cacheField name="[Measures].[Sum of category_percentage 2]" caption="Sum of category_percentage 2" numFmtId="0" hierarchy="35" level="32767"/>
+    <cacheField name="[Category_Percentage_NY].[category].[category]" caption="category" numFmtId="0" hierarchy="4" level="1">
+      <sharedItems count="6">
+        <s v="Apparel and Merchandise"/>
+        <s v="Art Supplies"/>
+        <s v="Books (General)"/>
+        <s v="Stationery and Supplies"/>
+        <s v="Technology &amp; Accessories"/>
+        <s v="Textbooks"/>
+      </sharedItems>
+    </cacheField>
+  </cacheFields>
+  <cacheHierarchies count="36">
+    <cacheHierarchy uniqueName="[Category_Percentage_CT].[store_id]" caption="store_id" attribute="1" defaultMemberUniqueName="[Category_Percentage_CT].[store_id].[All]" allUniqueName="[Category_Percentage_CT].[store_id].[All]" dimensionUniqueName="[Category_Percentage_CT]" displayFolder="" count="2" memberValueDatatype="20" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Category_Percentage_CT].[category]" caption="category" attribute="1" defaultMemberUniqueName="[Category_Percentage_CT].[category].[All]" allUniqueName="[Category_Percentage_CT].[category].[All]" dimensionUniqueName="[Category_Percentage_CT]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Category_Percentage_CT].[category_percentage]" caption="category_percentage" attribute="1" defaultMemberUniqueName="[Category_Percentage_CT].[category_percentage].[All]" allUniqueName="[Category_Percentage_CT].[category_percentage].[All]" dimensionUniqueName="[Category_Percentage_CT]" displayFolder="" count="2" memberValueDatatype="5" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Category_Percentage_NY].[store_id]" caption="store_id" attribute="1" defaultMemberUniqueName="[Category_Percentage_NY].[store_id].[All]" allUniqueName="[Category_Percentage_NY].[store_id].[All]" dimensionUniqueName="[Category_Percentage_NY]" displayFolder="" count="2" memberValueDatatype="20" unbalanced="0">
+      <fieldsUsage count="2">
+        <fieldUsage x="-1"/>
+        <fieldUsage x="0"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Category_Percentage_NY].[category]" caption="category" attribute="1" defaultMemberUniqueName="[Category_Percentage_NY].[category].[All]" allUniqueName="[Category_Percentage_NY].[category].[All]" dimensionUniqueName="[Category_Percentage_NY]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0">
+      <fieldsUsage count="2">
+        <fieldUsage x="-1"/>
+        <fieldUsage x="2"/>
+      </fieldsUsage>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Category_Percentage_NY].[category_percentage]" caption="category_percentage" attribute="1" defaultMemberUniqueName="[Category_Percentage_NY].[category_percentage].[All]" allUniqueName="[Category_Percentage_NY].[category_percentage].[All]" dimensionUniqueName="[Category_Percentage_NY]" displayFolder="" count="2" memberValueDatatype="5" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month].[Month]" caption="Month" attribute="1" time="1" defaultMemberUniqueName="[Month_by_Month].[Month].[All]" allUniqueName="[Month_by_Month].[Month].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="2" memberValueDatatype="7" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month].[Total_Revenue]" caption="Total_Revenue" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Total_Revenue].[All]" allUniqueName="[Month_by_Month].[Total_Revenue].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="2" memberValueDatatype="5" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month].[Month (Year)]" caption="Month (Year)" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Month (Year)].[All]" allUniqueName="[Month_by_Month].[Month (Year)].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month].[Month (Quarter)]" caption="Month (Quarter)" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Month (Quarter)].[All]" allUniqueName="[Month_by_Month].[Month (Quarter)].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month].[Month (Month)]" caption="Month (Month)" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Month (Month)].[All]" allUniqueName="[Month_by_Month].[Month (Month)].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month]" caption="month" attribute="1" time="1" defaultMemberUniqueName="[Month_by_Month_CT].[month].[All]" allUniqueName="[Month_by_Month_CT].[month].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="2" memberValueDatatype="7" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_CT].[total_revenue]" caption="total_revenue" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[total_revenue].[All]" allUniqueName="[Month_by_Month_CT].[total_revenue].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="2" memberValueDatatype="5" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month (Year)]" caption="month (Year)" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[month (Year)].[All]" allUniqueName="[Month_by_Month_CT].[month (Year)].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month (Quarter)]" caption="month (Quarter)" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[month (Quarter)].[All]" allUniqueName="[Month_by_Month_CT].[month (Quarter)].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month (Month)]" caption="month (Month)" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[month (Month)].[All]" allUniqueName="[Month_by_Month_CT].[month (Month)].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month]" caption="month" attribute="1" time="1" defaultMemberUniqueName="[Month_by_Month_NY].[month].[All]" allUniqueName="[Month_by_Month_NY].[month].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="2" memberValueDatatype="7" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_NY].[total_revenue]" caption="total_revenue" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[total_revenue].[All]" allUniqueName="[Month_by_Month_NY].[total_revenue].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="2" memberValueDatatype="5" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month (Year)]" caption="month (Year)" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[month (Year)].[All]" allUniqueName="[Month_by_Month_NY].[month (Year)].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month (Quarter)]" caption="month (Quarter)" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[month (Quarter)].[All]" allUniqueName="[Month_by_Month_NY].[month (Quarter)].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month (Month)]" caption="month (Month)" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[month (Month)].[All]" allUniqueName="[Month_by_Month_NY].[month (Month)].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="2" memberValueDatatype="130" unbalanced="0"/>
+    <cacheHierarchy uniqueName="[Month_by_Month].[Month (Month Index)]" caption="Month (Month Index)" attribute="1" defaultMemberUniqueName="[Month_by_Month].[Month (Month Index)].[All]" allUniqueName="[Month_by_Month].[Month (Month Index)].[All]" dimensionUniqueName="[Month_by_Month]" displayFolder="" count="2" memberValueDatatype="20" unbalanced="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_CT].[month (Month Index)]" caption="month (Month Index)" attribute="1" defaultMemberUniqueName="[Month_by_Month_CT].[month (Month Index)].[All]" allUniqueName="[Month_by_Month_CT].[month (Month Index)].[All]" dimensionUniqueName="[Month_by_Month_CT]" displayFolder="" count="2" memberValueDatatype="20" unbalanced="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Month_by_Month_NY].[month (Month Index)]" caption="month (Month Index)" attribute="1" defaultMemberUniqueName="[Month_by_Month_NY].[month (Month Index)].[All]" allUniqueName="[Month_by_Month_NY].[month (Month Index)].[All]" dimensionUniqueName="[Month_by_Month_NY]" displayFolder="" count="2" memberValueDatatype="20" unbalanced="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__XL_Count Month_by_Month_NY]" caption="__XL_Count Month_by_Month_NY" measure="1" displayFolder="" measureGroup="Month_by_Month_NY" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__XL_Count Month_by_Month_CT]" caption="__XL_Count Month_by_Month_CT" measure="1" displayFolder="" measureGroup="Month_by_Month_CT" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__XL_Count Month_by_Month]" caption="__XL_Count Month_by_Month" measure="1" displayFolder="" measureGroup="Month_by_Month" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__XL_Count Category_Percentage_CT]" caption="__XL_Count Category_Percentage_CT" measure="1" displayFolder="" measureGroup="Category_Percentage_CT" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__XL_Count Category_Percentage_NY]" caption="__XL_Count Category_Percentage_NY" measure="1" displayFolder="" measureGroup="Category_Percentage_NY" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[__No measures defined]" caption="__No measures defined" measure="1" displayFolder="" count="0" hidden="1"/>
+    <cacheHierarchy uniqueName="[Measures].[Sum of total_revenue 2]" caption="Sum of total_revenue 2" measure="1" displayFolder="" measureGroup="Month_by_Month_NY" count="0" hidden="1">
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="17"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[Sum of total_revenue]" caption="Sum of total_revenue" measure="1" displayFolder="" measureGroup="Month_by_Month_CT" count="0" hidden="1">
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="12"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[Sum of Total_Revenue 3]" caption="Sum of Total_Revenue 3" measure="1" displayFolder="" measureGroup="Month_by_Month" count="0" hidden="1">
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="7"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[Sum of category_percentage]" caption="Sum of category_percentage" measure="1" displayFolder="" measureGroup="Category_Percentage_CT" count="0" hidden="1">
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="2"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[Sum of store_id]" caption="Sum of store_id" measure="1" displayFolder="" measureGroup="Category_Percentage_CT" count="0" hidden="1">
+      <extLst>
+        <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
+          <x15:cacheHierarchy aggregatedColumn="0"/>
+        </ext>
+      </extLst>
+    </cacheHierarchy>
+    <cacheHierarchy uniqueName="[Measures].[Sum of category_percentage 2]" caption="Sum of category_percentage 2" measure="1" displayFolder="" measureGroup="Category_Percentage_NY" count="0" oneField="1" hidden="1">
+      <fieldsUsage count="1">
+        <fieldUsage x="1"/>
+      </fieldsUsage>
       <extLst>
         <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{B97F6D7D-B522-45F9-BDA1-12C45D357490}">
           <x15:cacheHierarchy aggregatedColumn="5"/>
@@ -17144,7 +18526,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E55EDF3E-0C25-4B31-8626-36D4AA832175}" name="PivotTable3" cacheId="395" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="13">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E55EDF3E-0C25-4B31-8626-36D4AA832175}" name="PivotTable3" cacheId="845" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="13">
   <location ref="D2:E7" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1">
@@ -17154,7 +18536,7 @@
     </pivotField>
     <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0">
       <items count="1">
-        <item x="0" e="0"/>
+        <item s="1" x="0" e="0"/>
       </items>
     </pivotField>
     <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0">
@@ -17202,28 +18584,28 @@
     <dataField name="Sum of total_revenue" fld="4" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="8">
-    <format dxfId="508">
+    <format dxfId="732">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="507">
+    <format dxfId="731">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="506">
+    <format dxfId="730">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="505">
+    <format dxfId="729">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="504">
+    <format dxfId="728">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="503">
+    <format dxfId="727">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="502">
+    <format dxfId="726">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="501">
+    <format dxfId="725">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -17287,11 +18669,7 @@
     <pivotHierarchy dragToData="1"/>
     <pivotHierarchy multipleItemSelectionAllowed="1" dragToData="1"/>
     <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy multipleItemSelectionAllowed="1" dragToData="1">
-      <members count="1" level="1">
-        <member name="[Month_by_Month_CT].[month (Month)].&amp;[Jun]"/>
-      </members>
-    </pivotHierarchy>
+    <pivotHierarchy multipleItemSelectionAllowed="1" dragToData="1"/>
     <pivotHierarchy dragToData="1"/>
     <pivotHierarchy dragToData="1"/>
     <pivotHierarchy dragToData="1"/>
@@ -17337,7 +18715,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{11C04DB6-74F1-419C-9320-B90911B6D254}" name="PivotTable2" cacheId="305" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="40">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{11C04DB6-74F1-419C-9320-B90911B6D254}" name="PivotTable2" cacheId="848" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="40">
   <location ref="D13:E18" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1">
@@ -17400,28 +18778,28 @@
     <dataField name="Sum of total_revenue" fld="4" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="8">
-    <format dxfId="499">
+    <format dxfId="723">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="498">
+    <format dxfId="722">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="497">
+    <format dxfId="721">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="496">
+    <format dxfId="720">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="495">
+    <format dxfId="719">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="494">
+    <format dxfId="718">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="493">
+    <format dxfId="717">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="492">
+    <format dxfId="716">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -17514,7 +18892,11 @@
     <pivotHierarchy dragToData="1"/>
     <pivotHierarchy multipleItemSelectionAllowed="1" dragToData="1"/>
     <pivotHierarchy dragToData="1"/>
-    <pivotHierarchy multipleItemSelectionAllowed="1" dragToData="1"/>
+    <pivotHierarchy multipleItemSelectionAllowed="1" dragToData="1">
+      <members count="1" level="1">
+        <member name="[Month_by_Month_NY].[month (Month)].&amp;[Jul]"/>
+      </members>
+    </pivotHierarchy>
     <pivotHierarchy dragToData="1"/>
     <pivotHierarchy dragToData="1"/>
     <pivotHierarchy dragToData="1"/>
@@ -17555,7 +18937,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C20E3E4A-2C2D-4515-8A39-76BB4333DF00}" name="PivotTable4" cacheId="518" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="16">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C20E3E4A-2C2D-4515-8A39-76BB4333DF00}" name="PivotTable4" cacheId="809" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="16">
   <location ref="D3:E8" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
@@ -17674,28 +19056,28 @@
     <dataField name="Sum of Total_Revenue" fld="0" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="8">
-    <format dxfId="16">
+    <format dxfId="704">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="17">
+    <format dxfId="705">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="18">
+    <format dxfId="706">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="19">
+    <format dxfId="707">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="20">
+    <format dxfId="708">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="21">
+    <format dxfId="709">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="22">
+    <format dxfId="710">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="23">
+    <format dxfId="711">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -17829,7 +19211,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{79054FA0-DBD8-4C88-8654-7D3990F87F77}" name="PivotTable1" cacheId="407" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="13">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{79054FA0-DBD8-4C88-8654-7D3990F87F77}" name="PivotTable1" cacheId="851" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="13">
   <location ref="E3:G11" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1">
@@ -18069,7 +19451,7 @@
             <x v="2"/>
           </reference>
           <reference field="2" count="1" selected="0">
-            <x v="4"/>
+            <x v="5"/>
           </reference>
         </references>
       </pivotArea>
@@ -18084,7 +19466,7 @@
             <x v="2"/>
           </reference>
           <reference field="2" count="1" selected="0">
-            <x v="5"/>
+            <x v="4"/>
           </reference>
         </references>
       </pivotArea>
@@ -18189,7 +19571,7 @@
             <x v="3"/>
           </reference>
           <reference field="2" count="1" selected="0">
-            <x v="4"/>
+            <x v="5"/>
           </reference>
         </references>
       </pivotArea>
@@ -18204,7 +19586,7 @@
             <x v="3"/>
           </reference>
           <reference field="2" count="1" selected="0">
-            <x v="5"/>
+            <x v="4"/>
           </reference>
         </references>
       </pivotArea>
@@ -18309,7 +19691,7 @@
             <x v="4"/>
           </reference>
           <reference field="2" count="1" selected="0">
-            <x v="4"/>
+            <x v="5"/>
           </reference>
         </references>
       </pivotArea>
@@ -18324,7 +19706,7 @@
             <x v="4"/>
           </reference>
           <reference field="2" count="1" selected="0">
-            <x v="5"/>
+            <x v="4"/>
           </reference>
         </references>
       </pivotArea>
@@ -18429,7 +19811,7 @@
             <x v="5"/>
           </reference>
           <reference field="2" count="1" selected="0">
-            <x v="4"/>
+            <x v="5"/>
           </reference>
         </references>
       </pivotArea>
@@ -18444,7 +19826,7 @@
             <x v="5"/>
           </reference>
           <reference field="2" count="1" selected="0">
-            <x v="5"/>
+            <x v="4"/>
           </reference>
         </references>
       </pivotArea>
@@ -18540,7 +19922,7 @@
             <x v="0"/>
           </reference>
           <reference field="2" count="1" selected="0">
-            <x v="4"/>
+            <x v="5"/>
           </reference>
         </references>
       </pivotArea>
@@ -18552,7 +19934,7 @@
             <x v="0"/>
           </reference>
           <reference field="2" count="1" selected="0">
-            <x v="5"/>
+            <x v="4"/>
           </reference>
         </references>
       </pivotArea>
@@ -18668,7 +20050,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C5BCED0D-BD63-4200-8981-6686C5C2DBCA}" name="PivotTable2" cacheId="419" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C5BCED0D-BD63-4200-8981-6686C5C2DBCA}" name="PivotTable2" cacheId="854" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
   <location ref="E3:G11" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField axis="axisCol" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1">
@@ -18867,7 +20249,7 @@
             <x v="0"/>
           </reference>
           <reference field="0" count="1" selected="0">
-            <x v="1"/>
+            <x v="0"/>
           </reference>
         </references>
       </pivotArea>
@@ -18879,7 +20261,7 @@
             <x v="0"/>
           </reference>
           <reference field="0" count="1" selected="0">
-            <x v="0"/>
+            <x v="1"/>
           </reference>
         </references>
       </pivotArea>
@@ -19060,7 +20442,7 @@
         </level>
       </levels>
       <selections count="1">
-        <selection n="[Month_by_Month_CT].[month (Month)].&amp;[Jun]"/>
+        <selection n="[Month_by_Month_CT].[month (Month)].&amp;[Sep]"/>
       </selections>
     </olap>
   </data>
@@ -19096,7 +20478,7 @@
         </level>
       </levels>
       <selections count="1">
-        <selection n="[Month_by_Month_NY].[month (Month)].[All]"/>
+        <selection n="[Month_by_Month_NY].[month (Month)].&amp;[Jul]"/>
       </selections>
     </olap>
   </data>
@@ -19256,7 +20638,7 @@
         </level>
       </levels>
       <selections count="1">
-        <selection n="[Category_Percentage_NY].[store_id].&amp;[851]"/>
+        <selection n="[Category_Percentage_NY].[store_id].&amp;[850]"/>
       </selections>
     </olap>
   </data>
@@ -19266,7 +20648,7 @@
 <file path=xl/slicers/slicer1.xml><?xml version="1.0" encoding="utf-8"?>
 <slicers xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
   <slicer name="month (Year) 1" xr10:uid="{56FEF96B-4AD0-4EE2-93E5-D4CB41895C55}" cache="Slicer_month__Year1" caption="Year" level="1" style="SlicerStyleLight6" rowHeight="251883"/>
-  <slicer name="month (Month)" xr10:uid="{788D754C-261B-46A7-BF70-482F06EE5B68}" cache="Slicer_month__Month" caption="Month" level="1" style="SlicerStyleLight6" rowHeight="251883"/>
+  <slicer name="month (Month)" xr10:uid="{788D754C-261B-46A7-BF70-482F06EE5B68}" cache="Slicer_month__Month" caption="Month" startItem="5" level="1" style="SlicerStyleLight6" rowHeight="251883"/>
 </slicers>
 </file>
 
@@ -19279,7 +20661,7 @@
 
 <file path=xl/slicers/slicer3.xml><?xml version="1.0" encoding="utf-8"?>
 <slicers xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
-  <slicer name="Month (Month) 2" xr10:uid="{0BAE40C7-4EC4-4FF1-929C-0192AC6858D6}" cache="Slicer_Month__Month2" caption=" Month" startItem="5" level="1" style="SlicerStyleLight6" rowHeight="251883"/>
+  <slicer name="Month (Month) 2" xr10:uid="{0BAE40C7-4EC4-4FF1-929C-0192AC6858D6}" cache="Slicer_Month__Month2" caption=" Month" level="1" style="SlicerStyleLight6" rowHeight="251883"/>
   <slicer name="Month (Year) 2" xr10:uid="{E0617DB9-8664-4DCA-9E76-9A1C3E35F0AD}" cache="Slicer_Month__Year2" caption="Year" level="1" style="SlicerStyleLight6" rowHeight="251883"/>
 </slicers>
 </file>
@@ -19300,7 +20682,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D6C9C94C-1CC7-4C97-AC20-872C5BD2F515}" name="Month_by_Month_CT" displayName="Month_by_Month_CT" ref="A1:B49" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:B49" xr:uid="{D6C9C94C-1CC7-4C97-AC20-872C5BD2F515}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{BE27E54F-B39F-4FBA-B965-22A9DEC4A798}" uniqueName="1" name="month" queryTableFieldId="1" dataDxfId="500"/>
+    <tableColumn id="1" xr3:uid="{BE27E54F-B39F-4FBA-B965-22A9DEC4A798}" uniqueName="1" name="month" queryTableFieldId="1" dataDxfId="724"/>
     <tableColumn id="2" xr3:uid="{813E2F6F-48CA-44A8-85D7-8D8F5BDDA1DD}" uniqueName="2" name="total_revenue" queryTableFieldId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -19308,10 +20690,10 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{AF376913-3285-41C5-97E5-2CBF051A5EA0}" name="Month_by_Month_NY" displayName="Month_by_Month_NY" ref="A1:B49" tableType="queryTable" totalsRowShown="0" headerRowDxfId="491">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{AF376913-3285-41C5-97E5-2CBF051A5EA0}" name="Month_by_Month_NY" displayName="Month_by_Month_NY" ref="A1:B49" tableType="queryTable" totalsRowShown="0" headerRowDxfId="715">
   <autoFilter ref="A1:B49" xr:uid="{AF376913-3285-41C5-97E5-2CBF051A5EA0}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{CA30B814-E434-45B5-886F-FD2A29F29689}" uniqueName="1" name="Month" queryTableFieldId="1" dataDxfId="490"/>
+    <tableColumn id="1" xr3:uid="{CA30B814-E434-45B5-886F-FD2A29F29689}" uniqueName="1" name="Month" queryTableFieldId="1" dataDxfId="714"/>
     <tableColumn id="2" xr3:uid="{61F5B8DD-1394-4143-9914-0ABFB5692836}" uniqueName="2" name="Total_Revenue" queryTableFieldId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -19319,10 +20701,10 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{362B4967-D55E-4E11-BE7F-11B7B2816DC4}" name="Month_by_Month" displayName="Month_by_Month" ref="A1:B49" tableType="queryTable" totalsRowShown="0" headerRowDxfId="510">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{362B4967-D55E-4E11-BE7F-11B7B2816DC4}" name="Month_by_Month" displayName="Month_by_Month" ref="A1:B49" tableType="queryTable" totalsRowShown="0" headerRowDxfId="734">
   <autoFilter ref="A1:B49" xr:uid="{362B4967-D55E-4E11-BE7F-11B7B2816DC4}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{EA185D14-DAC1-489F-A622-C8278CBD1C0B}" uniqueName="1" name="Month" queryTableFieldId="1" dataDxfId="509"/>
+    <tableColumn id="1" xr3:uid="{EA185D14-DAC1-489F-A622-C8278CBD1C0B}" uniqueName="1" name="Month" queryTableFieldId="1" dataDxfId="733"/>
     <tableColumn id="2" xr3:uid="{215FC225-09DD-47CA-8E8D-F5284C338924}" uniqueName="2" name="Total_Revenue" queryTableFieldId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -19334,7 +20716,7 @@
   <autoFilter ref="A1:C49" xr:uid="{0371816E-1392-4641-87A3-60DAF7B12802}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{7ECB9C14-9E1F-4908-84FB-F49B84EF8139}" uniqueName="1" name="store_id" queryTableFieldId="1"/>
-    <tableColumn id="2" xr3:uid="{799040DC-B12E-4D7D-80EB-AFF1C510B0EC}" uniqueName="2" name="category" queryTableFieldId="2" dataDxfId="489"/>
+    <tableColumn id="2" xr3:uid="{799040DC-B12E-4D7D-80EB-AFF1C510B0EC}" uniqueName="2" name="category" queryTableFieldId="2" dataDxfId="713"/>
     <tableColumn id="3" xr3:uid="{B5F4FB63-7D87-439B-8CE6-3A729F04B125}" uniqueName="3" name="category_percentage" queryTableFieldId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -19346,7 +20728,7 @@
   <autoFilter ref="A1:C73" xr:uid="{F919A6D9-E96E-49DC-AD4C-AA3CC0CFFD2E}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{DAEE007C-7DEC-4B84-9A85-21FC9D280D45}" uniqueName="1" name="store_id" queryTableFieldId="1"/>
-    <tableColumn id="2" xr3:uid="{55074EE6-F67F-4008-B204-F4A98BDAA45A}" uniqueName="2" name="category" queryTableFieldId="2" dataDxfId="488"/>
+    <tableColumn id="2" xr3:uid="{55074EE6-F67F-4008-B204-F4A98BDAA45A}" uniqueName="2" name="category" queryTableFieldId="2" dataDxfId="712"/>
     <tableColumn id="3" xr3:uid="{F34C736F-9180-4661-A337-ED57BB9BF597}" uniqueName="3" name="category_percentage" queryTableFieldId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -19727,7 +21109,7 @@
         <v>3</v>
       </c>
       <c r="E3" s="7">
-        <v>32008.85</v>
+        <v>30369.64</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -19741,7 +21123,7 @@
         <v>4</v>
       </c>
       <c r="E4" s="7">
-        <v>39754.07</v>
+        <v>49175.79</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
@@ -19755,7 +21137,7 @@
         <v>5</v>
       </c>
       <c r="E5" s="7">
-        <v>48142.95</v>
+        <v>44890.28</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
@@ -19769,7 +21151,7 @@
         <v>6</v>
       </c>
       <c r="E6" s="7">
-        <v>60671.67</v>
+        <v>71032.14</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
@@ -19783,7 +21165,7 @@
         <v>2</v>
       </c>
       <c r="E7" s="8">
-        <v>180577.54</v>
+        <v>195467.85</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
@@ -20270,7 +21652,7 @@
         <v>3</v>
       </c>
       <c r="E14" s="7">
-        <v>687382.03</v>
+        <v>56250.74</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
@@ -20284,7 +21666,7 @@
         <v>4</v>
       </c>
       <c r="E15" s="7">
-        <v>1044157.05</v>
+        <v>90818.8</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
@@ -20298,7 +21680,7 @@
         <v>5</v>
       </c>
       <c r="E16" s="7">
-        <v>1046676.37</v>
+        <v>89422.22</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
@@ -20312,7 +21694,7 @@
         <v>6</v>
       </c>
       <c r="E17" s="7">
-        <v>1552601.64</v>
+        <v>126976.23</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
@@ -20326,7 +21708,7 @@
         <v>2</v>
       </c>
       <c r="E18" s="8">
-        <v>4330817.09</v>
+        <v>363467.99</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
@@ -21797,7 +23179,7 @@
         <v>8</v>
       </c>
       <c r="F4">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="G4" t="s">
         <v>2</v>
@@ -21817,10 +23199,10 @@
         <v>16</v>
       </c>
       <c r="F5" s="7">
-        <v>4.2802E-2</v>
+        <v>4.4330000000000001E-2</v>
       </c>
       <c r="G5" s="7">
-        <v>4.2802E-2</v>
+        <v>4.4330000000000001E-2</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
@@ -21837,10 +23219,10 @@
         <v>18</v>
       </c>
       <c r="F6" s="7">
-        <v>3.6144000000000003E-2</v>
+        <v>3.5846999999999997E-2</v>
       </c>
       <c r="G6" s="7">
-        <v>3.6144000000000003E-2</v>
+        <v>3.5846999999999997E-2</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
@@ -21857,10 +23239,10 @@
         <v>20</v>
       </c>
       <c r="F7" s="7">
-        <v>1.8516000000000001E-2</v>
+        <v>1.6785999999999999E-2</v>
       </c>
       <c r="G7" s="7">
-        <v>1.8516000000000001E-2</v>
+        <v>1.6785999999999999E-2</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
@@ -21877,10 +23259,10 @@
         <v>15</v>
       </c>
       <c r="F8" s="7">
-        <v>1.7103E-2</v>
+        <v>1.4827999999999999E-2</v>
       </c>
       <c r="G8" s="7">
-        <v>1.7103E-2</v>
+        <v>1.4827999999999999E-2</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
@@ -21897,10 +23279,10 @@
         <v>19</v>
       </c>
       <c r="F9" s="7">
-        <v>0.70365100000000003</v>
+        <v>0.71080200000000004</v>
       </c>
       <c r="G9" s="7">
-        <v>0.70365100000000003</v>
+        <v>0.71080200000000004</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
@@ -21917,10 +23299,10 @@
         <v>17</v>
       </c>
       <c r="F10" s="7">
-        <v>0.181784</v>
+        <v>0.17740700000000001</v>
       </c>
       <c r="G10" s="7">
-        <v>0.181784</v>
+        <v>0.17740700000000001</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">

</xml_diff>